<commit_message>
fix menu as request 17-07
</commit_message>
<xml_diff>
--- a/output/bedrock_usage_log.xlsx
+++ b/output/bedrock_usage_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16394,6 +16394,3598 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-17T11:59:45.957609+00:00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>menu_api_call</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>arn:aws:bedrock:us-east-1:078805859846:inference-profile/us.anthropic.claude-sonnet-4-6</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>8159</v>
+      </c>
+      <c r="E21" t="n">
+        <v>5052</v>
+      </c>
+      <c r="F21" t="n">
+        <v>13211</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You are a structured data extraction engine.
+Task:
+Extract menu information from the provided menu image and convert it into structured JSON.
+Follow all rules strictly.
+--------------------------------------------------
+1. CATEGORY GROUPING
+--------------------------------------------------
+- Group all items under their respective category names.
+- Do not merge categories.
+- Do not skip any item.
+--------------------------------------------------
+2. SIZE HANDLING (Category-Level Sizes)
+--------------------------------------------------
+If a category contains size columns like R, M, L (or Small/Medium/Large or sml/lrg/Half/Full):
+    "lstInvSize": true
+Each item must use:
+    "sizes": { "R": price, "M": price, "L": price }
+    (use whatever size keys appear in the menu header, e.g. "S"/"M"/"L", "Half"/"Full", "sml"/"lrg")
+If a specific item in an R/M/L category is only available in one size (e.g. only M is priced):
+    Include only that size key in "sizes": { "M": price }
+    Do NOT force all size keys if they are blank or missing for that item.
+If a category has only one fixed size labeled "Only Medium" or similar:
+    "lstInvSize": false
+    "sizeType": "ONLY_MEDIUM"
+Use:
+    "price": value
+If a category has text-based size in the price itself (e.g. "sml 5.99/lrg 9.99"):
+    Treat as lstInvSize: true and extract the key-value pairs as sizes.
+If no size exists at all:
+    "lstInvSize": false
+    "sizeType": null
+--------------------------------------------------
+2B. MIXED SIZE CATEGORIES (PER-ITEM SIZES)
+--------------------------------------------------
+Some categories are otherwise flat, single-price categories, but ONE or A FEW individual items show their own inline size-based pricing directly in that item's row (e.g. "Milk Sm 2.25 ... Lrg 2.95" inside a category where every other item has one plain price).
+In this case:
+- Do NOT apply sizes to the whole category.
+- Leave the category as flat ("lstInvSize": false, "sizeType": null) if most items are plain-priced.
+- For the specific item(s) that show inline sizes, set:
+    "sizes": { "Sm": price, "Lrg": price }
+    (use whatever size labels appear next to that item, e.g. "Sm"/"Lrg", "Small"/"Large", "Half"/"Full")
+    "price": null
+- All other items in that category keep their normal single "price" value and empty "sizes": {}.
+Example:
+  Category "Beverages" (flat, single price):
+    - "Coffee"       → "price": 2.50, "sizes": {}
+    - "Milk"         → "price": null, "sizes": { "Sm": 2.25, "Lrg": 2.95 }
+--------------------------------------------------
+2C. PORTION-SIZE TIERS SHARING ONE DESCRIPTION (AVOID DUPLICATE ITEMS)
+--------------------------------------------------
+Some menus present ONE dish/description followed by several named portion-size tiers with different prices — shown as boxes, a header table, or inline labels (e.g. MINI/SENIOR/REGULAR/XLARGE, Small/Medium/Large/Family, Personal/Regular/Large, 4pcs/7pcs/12pcs/20pcs, Half/Full). This can happen regardless of visual layout — boxes, a table, or plain inline text — not just an inline R/M/L column next to the item row.
+DETECTION RULE (works for ANY menu style, ANY tier wording):
+Before finalizing items in a category, check: are you about to create MORE THAN ONE item that share the EXACT SAME (or near-identical) name/description and differ ONLY by a size/portion/quantity label and its price? If yes, STOP — merge them into ONE item instead.
+Rule:
+- Create exactly ONE item using the shared description.
+- "sizes": { "&lt;tier label 1&gt;": price, "&lt;tier label 2&gt;": price, ... } — use the exact tier labels/wording printed on the menu (e.g. "Mini", "Senior", "Regular", "XLarge", "4pcs", "7pcs").
+- "price": null (the price lives entirely in "sizes").
+- Do NOT create a separate item per tier, even if the tiers are printed in separate boxes/columns/callouts rather than a single row.
+This generalizes Section 2 to portion/quantity-tier wording beyond R/M/L, and applies to any category where one dish is offered at multiple named tiers.
+--------------------------------------------------
+3. PRICE FORMAT DETECTION
+--------------------------------------------------
+Before mapping prices to items or modifier options, parse prices using these rules:
+A) Single numeric price:
+   "120/-"   → 120
+   "120"     → 120
+   "$5.99"   → 5.99
+B) Two prices separated by "/" or " " (slash/space):
+   "140/- 160/-"   → [140, 160]
+   "140/160"       → [140, 160]
+   "5.99/lrg 9.99" → handled as sizes (see Section 2)
+C) Three or more prices — concatenated with "/-" or "/" or space:
+   "150/-160/-170/-"    → [150, 160, 170]
+   "150/160/170"        → [150, 160, 170]
+   "200/-220/-210/-"    → [200, 220, 210]
+D) Multi-line prices (prices split across two visual lines in the menu):
+   Concatenate all price tokens for that item row and map sequentially.
+   Example: first line "150/-160/-170/-", second line "170/-160/-"
+   → combined prices: [150, 160, 170, 170, 160]
+E) "MRP" price (no fixed price printed):
+   "price": null
+F) If price count and modifier option count mismatch:
+   Map sequentially. Assign 0 to any remaining options without a price.
+--------------------------------------------------
+4. ITEM-LEVEL MODIFIER DETECTION
+--------------------------------------------------
+If an item name contains option patterns such as:
+- (Veg/Non Veg)
+- (Veg / Non Veg)
+- (Paneer, Baby Corn, Mushroom, Gobi)
+- (Chicken, Prawn, Fish)
+- Any slash-separated or comma-separated values inside brackets
+Then treat this as ITEM-LEVEL MODIFIER.
+EXCEPTION — Single-label items: If the bracket contains only ONE value like "(Non Veg)" or "(Veg)" and the item has a single price, do NOT create a modifier. Simply strip the bracket and use the item name as-is with that single price.
+For all other bracket patterns, You MUST:
+A) Set category:
+   "lstInventoryModifiers": true
+B) Remove bracket content from item name.
+C) Create a separate modifier group per item:
+{
+  "groupName": "Item Name Modifiers",
+  "type": "modifier",
+  "lstInvSize": false,
+  "options": [
+    {
+      "name": "Option Name",
+      "price": 0,
+      "modifierGroup": null
+    }
+  ]
+}
+D) Price Mapping Rules (use Section 3 to parse prices first):
+Parse all prices from the item's price field, then map sequentially:
+   First price  → First modifier option
+   Second price → Second modifier option
+   Third price  → Third modifier option
+   ...and so on.
+If more options than prices: assign price 0 to remaining options.
+If more prices than options: map sequentially, ignore extras.
+E) Item structure when modifier exists:
+{
+  "name": "Item Name",
+  "description": null,
+  "sizes": {},
+  "price": null,
+  "modifierGroup": "Item Name Modifiers"
+}
+IMPORTANT:
+- Do NOT keep combined price at item level.
+- Move all pricing into modifier options.
+- EXCEPTION: if every option costs the SAME amount (i.e. the menu prints only ONE overall price and the choice doesn't change it), do NOT null the item price — see Section 4C instead.
+--------------------------------------------------
+4B. TEXTUAL CHOICE MODIFIER (NO BRACKETS)
+--------------------------------------------------
+Some items offer a choice between named options WITHOUT brackets, expressed as plain text such as:
+   "with Bacon, or Sausage Patties, or Bologna, or Liver Mush ... 8.95"
+   "with Ham or Links ... 9.25"
+   "choice of A, or B ... price"
+If an item's text lists two or more named choices (separated by commas and/or "or") introduced by words like "with" / "choice of" / "your choice of", AND different choice groups carry DIFFERENT prices (multi-tier pricing for the same base item), treat this as an ITEM-LEVEL MODIFIER using the same structure as Section 4:
+A) Set category: "lstInventoryModifiers": true
+B) Strip the choice text from the item name, keeping only the base item name (e.g. "Waffle").
+C) Create ONE modifier group for the item:
+{
+  "groupName": "Item Name Modifiers",
+  "type": "modifier",
+  "lstInvSize": false,
+  "options": [
+    { "name": "Choice A", "price": 0, "modifierGroup": null },
+    { "name": "Choice B", "price": 0, "modifierGroup": null }
+  ]
+}
+D) Split EACH individual choice name (comma/"or"-separated) within a price tier into its OWN modifier option, and assign that tier's price to every option within that tier.
+   Example: "with Bacon, or Sausage Patties, or Bologna, or Liver Mush ... 8.95 with Ham or Links ... 9.25"
+   → options: Bacon (8.95), Sausage Patties (8.95), Bologna (8.95), Liver Mush (8.95), Ham (9.25), Links (9.25)
+E) Item structure when this modifier exists:
+{
+  "name": "Waffle",
+  "description": null,
+  "sizes": {},
+  "price": null,
+  "modifierGroup": "Waffle Modifiers"
+}
+F) Do NOT trigger this rule (the multi-tier price split) for plain descriptive "choice of" text that has only ONE price for the whole item. Only trigger THIS rule (4B) when different choice groups map to DIFFERENT prices. When there is only ONE overall price, still capture the choice as a modifier — without splitting the price — per Section 4D.
+--------------------------------------------------
+4C. PRICE RETENTION RULE FOR NO-COST CHOICE MODIFIERS
+--------------------------------------------------
+Before nulling an item's "price" because a modifier group exists (Sections 4, 4B, 6, 7), check whether the modifier's options actually change the total price:
+- If EVERY option in the modifier group costs the SAME amount (including all being 0) — meaning the choice is just a variant/flavor/filling pick and the menu prints only ONE overall price for the item — then:
+    - KEEP the item's own "price" as that single printed price (do NOT null it).
+    - Set every option's "price" to 0 (the cost is already included in the item price).
+- Only set the item's "price" to null when different options carry genuinely DIFFERENT prices that change what the customer pays (a true upcharge/price-tier modifier, as in Section 4B).
+This rule applies globally to item-level (4/4B), category-level (6), and shared category-level (7) modifiers — never lose the printed price of an item just because it also offers a same-price choice.
+Example: "Pie Special — ALL £11.75 — Choose from: Steak, Meat &amp; Potato, Cheese &amp; Onion, Meat Pie, Steak Pudding" → "price": 11.75 (kept), every filling option priced 0.
+--------------------------------------------------
+4D. SINGLE-PRICE CHOICE MODIFIER (FLAT ALTERNATIVES, NO PRICE SPLIT)
+--------------------------------------------------
+Some items or categories list several named alternatives (flavors, fillings, proteins, sauces, toppings, etc. — separated by commas/"or"/newlines) where the menu prints only ONE overall price (no per-choice price difference). Examples: "Pie Special — ALL £11.75 — Choose from: Steak, Meat &amp; Potato, Cheese &amp; Onion, Meat Pie, Steak Pudding" or "Crispy Shredded Chicken — Choose a flavour! Plain, Salt &amp; Pepper or Salt &amp; Chilli — £11.75".
+For this pattern:
+A) Keep the item's own "price" as the single printed price (per Section 4C — do NOT null it).
+B) Still capture every named alternative as a modifier — do NOT drop the choice information just because there's no price split. Wrap ALL alternatives under ONE modifier group named after what is being chosen (e.g. "Choice of Filling", "Choice of Flavour"), using the NESTED MODIFIER GROUP mechanism from Section 8:
+   - The item's (or category's) own modifierGroup has exactly ONE option — the wrapping choice name (e.g. "Choice of Filling") — whose own "modifierGroup" field points to a second modifierGroups entry.
+   - That second modifierGroups entry lists every named alternative (Steak, Meat &amp; Potato, Cheese &amp; Onion, ...) as its options, each "price": 0.
+C) Do NOT create one separate top-level modifier per alternative (e.g. do NOT create 5 separate sibling groups named "Steak", "Meat &amp; Potato", etc. each with no sub-options) — every alternative must be a nested option inside the ONE wrapping group.
+D) This applies whether the choice is described at item level (Section 4) or for an entire category (Section 6) — use the same item/category "modifierGroup" assignment mechanics already defined in those sections, just wrap the flat list per this rule instead of exploding it.
+--------------------------------------------------
+5. MIXED MODIFIER CATEGORIES
+--------------------------------------------------
+If a category has SOME items with bracket modifiers and SOME items without:
+- Apply item-level modifiers ONLY to items that have bracket patterns.
+- Items without brackets remain as plain items with a direct price.
+- Set category: "lstInventoryModifiers": true (because at least one item has a modifier).
+Example:
+  - "Veg Noodle" with price 120 → plain item, no modifier
+  - "Mix Noodle (Veg/Non Veg)" with prices 140/160 → item-level modifier
+--------------------------------------------------
+6. CATEGORY-LEVEL MODIFIER DETECTION
+--------------------------------------------------
+If a modifier section applies to ALL items within a single category
+(e.g., Half/Full, Regular/Large, Veg/Non Veg for whole category),
+Then:
+A) Set:
+   "lstInventoryModifiers": true
+B) Create ONE modifier group for that category:
+{
+  "groupName": "Category Name Modifiers",
+  "type": "modifier",
+  "lstInvSize": false,
+  "options": [
+    {
+      "name": "Option Name",
+      "price": 0,
+      "modifierGroup": null
+    }
+  ]
+}
+C) Assign:
+   "modifierGroup": "Category Name Modifiers"
+D) Map prices sequentially per item if multiple prices exist.
+E) Do NOT create separate modifier groups per item.
+--------------------------------------------------
+6B. CATEGORY-WIDE INCLUDED SERVING NOTE (NO PRICE, MULTIPLE CHOICE GROUPS)
+--------------------------------------------------
+Some categories carry a shared note — a header or footer line positioned ABOVE/BELOW the item list rather than inside any single item's own row/price cell — describing what EVERY item in that category is served with. Examples:
+   "Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit."
+   "Two Eggs* served with Home Fries or Grits or Hash Browns, and Toast or Biscuit."
+Treat this as a CATEGORY-LEVEL MODIFIER (Section 6) with these specifics:
+A) No price change: the note is already included in every item's own price. Follow the price-retention rule (Section 4C) — keep each item's own printed "price", and price every modifier option 0.
+B) The note may describe MORE THAN ONE independent choice group joined by "and"/commas (e.g. a side choice AND a separate bread choice). Do NOT flatten these into one list. Create ONE modifier group per distinct choice category (e.g. "Choose Side", "Choose Bread"), each wrapped using the SAME nested-wrap mechanism as Section 4D:
+   - The category's own "modifierGroup" points to ONE modifierGroups entry whose "options" are the wrapping choice names ("Choose Side", "Choose Bread", etc.), each option's own "modifierGroup" pointing to a further modifierGroups entry holding the actual named choices (e.g. Hash Browns/Grits/Home Fries under "Choose Side"; Toast/Biscuit under "Choose Bread").
+C) Apply this "modifierGroup" at the CATEGORY level (per Section 6) so it covers EVERY item in the category — do not attach it per item.
+D) Copy the shared note text into EACH item's own "description" field as well (combine with any item-specific description text if present), so no item is left with a blank description just because its serving note lives outside the item row.
+E) If the identical (or near-identical) shared note/choice set recurs across MULTIPLE categories (e.g. the same Hash Browns/Grits/Home Fries + Toast/Biscuit choice appears under an omelette category, a steak-and-eggs category, and a fish category), do NOT rebuild duplicate modifier groups per category. Define the wrapping group and its nested choice groups ONCE in "modifierGroups", and assign that SAME "modifierGroup" name to every matching category — this qualifies as a SHARED CATEGORY-LEVEL MODIFIER (Section 7) even without an explicitly named header like "Extra Topping."
+F) This pattern is not limited to breakfast sides — any cuisine/menu style where a whole category shares an included, no-extra-cost choice note (e.g. "Served with rice or naan", "Includes soup or salad", "Comes with fries or side salad") follows this same rule.
+--------------------------------------------------
+7. SHARED CATEGORY-LEVEL MODIFIER (MULTIPLE CATEGORIES)
+--------------------------------------------------
+If a separate section exists such as:
+- Extra Topping
+- Add Ons
+- Upgrade Options
+- Additional Toppings
+...OR a repeated shared serving note without a distinct named header (see Section 6B-E, e.g. the same "served with X or Y" choice printed under several categories)
+And it clearly applies to multiple categories
+(e.g., American Veg Pizza, Desi Veg Pizza, Italian Veg Pizza),
+Then treat it as SHARED CATEGORY-LEVEL MODIFIER.
+You MUST:
+A) Create ONE shared modifier group:
+{
+  "groupName": "Extra Topping",
+  "type": "modifier",
+  "lstInvSize": true/false,
+  "options": [
+    {
+      "name": "Extra Cheese",
+      "price": 0,
+      "prices": { "R": 40, "M": 60, "L": 90 },
+      "modifierGroup": null
+    }
+  ]
+}
+B) If modifier pricing depends on size (R/M/L):
+   "lstInvSize": true
+   Use:
+      "prices": { "R": value, "M": value, "L": value }
+C) If single price:
+   "lstInvSize": false
+   Use: "price": value
+D) Assign this modifier group to ALL applicable categories:
+{
+  "category": "American Veg Pizza",
+  "lstInventoryModifiers": true,
+  "modifierGroup": "Extra Topping"
+}
+E) Do NOT duplicate shared modifier groups.
+--------------------------------------------------
+8. NESTED MODIFIER GROUP (MODIFIER INSIDE MODIFIER)
+--------------------------------------------------
+If a modifier option itself contains selectable options visible in the menu
+(example: Extra Cheese → shows sub-list: Mozzarella, Cheddar, Parmesan)
+Then treat this as a NESTED MODIFIER GROUP.
+You MUST:
+A) Create a separate modifier group for the inner modifier:
+{
+  "groupName": "Extra Cheese Type",
+  "type": "modifier",
+  "lstInvSize": false,
+  "options": [
+    {
+      "name": "Mozzarella",
+      "price": 0,
+      "modifierGroup": null
+    },
+    {
+      "name": "Cheddar",
+      "price": 0,
+      "modifierGroup": null
+    }
+  ]
+}
+B) Attach this nested group to the parent modifier option:
+{
+  "name": "Extra Cheese",
+  "price": 40,
+  "modifierGroup": "Extra Cheese Type"
+}
+C) Nested modifier must NOT duplicate pricing unless explicitly shown.
+D) Nested modifiers can exist under:
+   Item-level modifier
+   Category-level modifier
+   Shared category-level modifier
+E) Maintain hierarchy strictly:
+   Category → Item → Modifier → Nested Modifier
+--------------------------------------------------
+9. ITEMS WITHOUT MODIFIERS
+--------------------------------------------------
+If item has:
+- No size
+- No modifier
+- No variation
+Then:
+{
+  "name": "",
+  "description": null,
+  "sizes": {},
+  "price": value,
+  "modifierGroup": null
+}
+If price is MRP (no fixed price printed):
+  "price": null
+And category:
+    "lstInventoryModifiers": false
+--------------------------------------------------
+9B. ITEM TYPE DETECTION (PRODUCT VS COMBO)
+--------------------------------------------------
+Every item must be classified with an "itemType" field:
+- Set "itemType": "combo" if:
+    - The item name or its category name contains bundle wording such as "Combo", "Meal", "Set Meal", "Value Meal", "Platter Combo", or similar, OR
+    - The item explicitly bundles multiple separate components into one fixed price (e.g. "Waffle Combo w/ Two Eggs, Bacon or Sausage, and Toast").
+- Otherwise set "itemType": "product" (default for all normal, non-bundled menu items).
+For "itemType": "combo" items:
+   - Do NOT use "modifierGroup" / "sizes" for the combo's bundled components — use "comboGroups" instead (see Section 9C).
+   - "sizes" stays {} and "modifierGroup" stays null on the item, unless the combo itself is separately offered in multiple sizes.
+   - "price" is the combo's own total price (e.g. 11.45).
+For "itemType": "product" items, "comboGroups" stays [] (unused) and normal "sizes" / "modifierGroup" rules (Sections 2, 2B, 4, 4B, 6, 7) apply as usual.
+CONSISTENCY RULE: If the exact same item name/description text appears in more than one category/section of the menu (e.g. the same combo listed both in a "Combos" section and again in a "Mains" section), classify and structure it IDENTICALLY everywhere it appears — same "itemType", same "sizes"/"comboGroups"/"modifierGroup" breakdown, same level of detail. Base classification purely on the item's own text — never on which category box or section it happens to be printed in.
+--------------------------------------------------
+9C. COMBO COMPONENT BREAKDOWN ("comboGroups")
+--------------------------------------------------
+For every "itemType": "combo" item, break down its bundled components into "comboGroups". Read the combo's full text (e.g. "Two Eggs* with choice of Bacon, Sausage Patties, Liver Mush or Beef Bologna, served with Grits, Hash Browns, or Home Fries, and a Waffle") and identify each distinct component:
+A) FIXED / INCLUDED component (no choice, always part of the combo, e.g. "Two Eggs", "a Waffle", "Toast or Biscuit" if only one is always given):
+   - One comboGroup per fixed component.
+   - "isInclude": true
+   - "minQty": 1, "maxQty": 1
+   - Exactly ONE option in "options", price 0 (already covered by the combo price) unless the menu prints an explicit extra charge.
+B) CHOICE component (customer selects one from a named list, e.g. "choice of Bacon, Sausage Patties, Liver Mush or Beef Bologna"):
+   - One comboGroup per distinct choice category (e.g. "Choice of Meat", "Choice of Side", "Choice of Bread").
+   - "isInclude": false
+   - "minQty": 1, "maxQty": 1 (or higher "maxQty" only if the menu explicitly allows selecting more than one)
+   - Split each named choice (comma/"or"-separated) into its own option, price 0 unless the menu shows an explicit add-on charge for that specific choice.
+C) Name each comboGroup by what it represents (e.g. "Eggs", "Choice of Meat", "Choice of Side"), not generically.
+D) Combine the combo's full bundled text into one natural-language sentence in the item's "description" field (e.g. "Two eggs with choice of bacon, sausage patties, liver mush or beef bologna, served with grits, hash browns, or home fries and a waffle.").
+E) Structure:
+{
+  "name": "Super Waffle Combo",
+  "description": "Two eggs with choice of bacon, sausage patties, liver mush or beef bologna, served with grits or hash browns or home fries and a waffle combo.",
+  "sizes": {},
+  "price": 11.45,
+  "modifierGroup": null,
+  "itemType": "combo",
+  "comboGroups": [
+    {
+      "groupName": "Eggs",
+      "isInclude": true,
+      "minQty": 1,
+      "maxQty": 1,
+      "options": [ { "name": "Two Eggs", "price": 0 } ]
+    },
+    {
+      "groupName": "Choice of Meat",
+      "isInclude": false,
+      "minQty": 1,
+      "maxQty": 1,
+      "options": [
+        { "name": "Bacon", "price": 0 },
+        { "name": "Sausage Patties", "price": 0 },
+        { "name": "Liver Mush", "price": 0 },
+        { "name": "Beef Bologna", "price": 0 }
+      ]
+    },
+    {
+      "groupName": "Choice of Side",
+      "isInclude": false,
+      "minQty": 1,
+      "maxQty": 1,
+      "options": [
+        { "name": "Grits", "price": 0 },
+        { "name": "Hash Browns", "price": 0 },
+        { "name": "Home Fries", "price": 0 }
+      ]
+    }
+  ]
+}
+F) This applies to ANY combo menu, not just breakfast combos — pizza combos, burger combos, thali/set-meal combos, etc. Always decompose into "fixed inclusion" groups vs "choice" groups using rules A and B above, regardless of cuisine or category name.
+--------------------------------------------------
+10. MODIFIER PRIORITY RULE
+--------------------------------------------------
+1. If modifier applies only to one item → Item-Level Modifier.
+2. If modifier applies to entire category → Category-Level Modifier.
+3. If modifier applies to multiple categories → Shared Category-Level Modifier.
+4. If modifier option has sub-options → Nested Modifier Group.
+5. Never duplicate modifier groups.
+--------------------------------------------------
+11. FINAL STRUCTURE (STRICT FORMAT)
+--------------------------------------------------
+Return ONLY this JSON structure:
+{
+  "categories": [
+    {
+      "category": "",
+      "lstInvSize": true/false,
+      "lstInventoryModifiers": true/false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "",
+          "description": null,
+          "sizes": {},
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    }
+  ],
+  "modifierGroups": [
+    {
+      "groupName": "",
+      "type": "modifier",
+      "lstInvSize": true/false,
+      "options": [
+        {
+          "name": "",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        }
+      ]
+    }
+  ]
+}
+--------------------------------------------------
+12. STRICT RULES
+--------------------------------------------------
+- Do not skip any item.
+- Keep prices as numbers only (no "/- " suffix, no currency symbols).
+- Remove brackets and their content from item names.
+- Do not duplicate modifier groups.
+- Do not leave price at item level if a modifier group exists, UNLESS every option in that modifier group is equal-price/no-cost (see Section 4C) — in that case keep the item price and set option prices to 0.
+- If price count and modifier count mismatch, map sequentially; assign 0 to unpaired options.
+- Nested modifiers must reference parent modifier correctly.
+- If a field is not applicable, set it to null (NOT empty string "").
+- "sizeType" must be null unless it is "ONLY_MEDIUM".
+- "modifierGroup" at category or item level must be null when not applicable.
+- "prices" field in modifier options must be {} (empty object) when not applicable.
+- "itemType" must be "product" for every regular item, and "combo" only for bundled/combo items (see Section 9B).
+- "comboGroups" must be [] for "product" items, and fully populated (fixed + choice groups, see Section 9C) for "combo" items.
+- Do not create multiple items in a category that share the same name/description and differ only by a size/portion tier label — merge into one item with "sizes" instead (see Section 2C).
+- If the same item text appears in more than one category, classify and structure it identically everywhere (see Section 9B consistency rule).
+- Do not leave "description" blank or skip modifiers just because a category's serving note (e.g. "served with X or Y, and A or B") sits outside the item row — apply it to every item in the category per Section 6B.
+- Return ONLY valid JSON.
+- Do NOT add explanations.
+- Do NOT use markdown.
+- Do not miss any itam details recheck and found any things is missing add the item proper as per rule
+</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>```json
+{
+  "categories": [
+    {
+      "category": "Omelettes",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": "Omelettes Serving Choice",
+      "items": [
+        {
+          "name": "Ham &amp; Cheese Omelette",
+          "description": "Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit",
+          "sizes": {},
+          "price": 9.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Sausage &amp; Cheese Omelette",
+          "description": "Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit",
+          "sizes": {},
+          "price": 9.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Cheese Omelette",
+          "description": "Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit",
+          "sizes": {},
+          "price": 8.45,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Mushroom &amp; Cheese Omelette",
+          "description": "Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit",
+          "sizes": {},
+          "price": 9.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Western Omelette",
+          "description": "A traditional western omelette with ham, green peppers, chopped onions and a blend of cheeses. Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit",
+          "sizes": {},
+          "price": 10.45,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Spanish Omelette",
+          "description": "Diced onions, tomatoes, ham and melted cheeses smothered with our favorite Spanish sauce. Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit",
+          "sizes": {},
+          "price": 10.45,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Turkey &amp; Cheese Omelette",
+          "description": "Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit",
+          "sizes": {},
+          "price": 9.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Vegetarian Omelette",
+          "description": "Mushrooms, onions, green peppers and tomatoes topped with a blend of cheeses. Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit",
+          "sizes": {},
+          "price": 9.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Farmer's Omelette",
+          "description": "Hickory smoked sausage with onions, peppers tomatoes and a blend of cheeses. Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit",
+          "sizes": {},
+          "price": 10.45,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Bacon and Cheese Omelette",
+          "description": "Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit",
+          "sizes": {},
+          "price": 9.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Greek Omelette",
+          "description": "Mediterranean feta cheese, tomatoes, Kalamata olives, and chopped onions. Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit",
+          "sizes": {},
+          "price": 10.45,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "The Sizzling Steak",
+          "description": "Grilled chunks of steak, mixed with peppers, onions and mushrooms, topped with a blend of cheeses. Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit",
+          "sizes": {},
+          "price": 11.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Supreme Chicken Omelette",
+          "description": "Marinated grilled chunks of chicken, onions, peppers and mushrooms, topped with a blend of cheeses. Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit",
+          "sizes": {},
+          "price": 11.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "The Famous Gyro Omelette",
+          "description": "Sliced mixture of lamb and beef with onions and tomatoes, sprinkled with feta cheese. Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit",
+          "sizes": {},
+          "price": 10.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Spinach &amp; Feta Cheese Omelette",
+          "description": "Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit",
+          "sizes": {},
+          "price": 10.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "10oz. Steak &amp; Eggs",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": "Omelettes Serving Choice",
+      "items": [
+        {
+          "name": "Rib Eye - Choice",
+          "description": "Two Eggs* served with Home Fries or Grits or Hash Browns, and Toast or Biscuit",
+          "sizes": {},
+          "price": 19.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Two Pork Chops - Center Cut",
+          "description": "Two Eggs* served with Home Fries or Grits or Hash Browns, and Toast or Biscuit",
+          "sizes": {},
+          "price": 13.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Chicken Breast - Grilled Fresh",
+          "description": "Two Eggs* served with Home Fries or Grits or Hash Browns, and Toast or Biscuit",
+          "sizes": {},
+          "price": 13.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Fish &amp; Grits",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": "Omelettes Serving Choice",
+      "items": [
+        {
+          "name": "Salmon Steak - Fresh Hand Cut",
+          "description": "Two Eggs* served with Home Fries or Grits or Hash Browns, and Toast or Biscuit",
+          "sizes": {},
+          "price": 16.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Fried Fillet of Flounder",
+          "description": "Two Eggs* served with Home Fries or Grits or Hash Browns, and Toast or Biscuit",
+          "sizes": {},
+          "price": 12.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Fried Jumbo Shrimp",
+          "description": "Two Eggs* served with Home Fries or Grits or Hash Browns, and Toast or Biscuit",
+          "sizes": {},
+          "price": 13.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Salmon Cakes - Homemade",
+          "description": "Two Eggs* served with Home Fries or Grits or Hash Browns, and Toast or Biscuit",
+          "sizes": {},
+          "price": 11.25,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Fried Fillet of Perch",
+          "description": "Two Eggs* served with Home Fries or Grits or Hash Browns, and Toast or Biscuit",
+          "sizes": {},
+          "price": 12.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Belgian Waffles",
+      "lstInvSize": false,
+      "lstInventoryModifiers": true,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Plain Waffle with Butter and Syrup",
+          "description": null,
+          "sizes": {},
+          "price": 6.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Waffle",
+          "description": null,
+          "sizes": {},
+          "price": null,
+          "modifierGroup": "Waffle Meat Modifiers",
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Add Strawberry or Blueberry Topping &amp; Whipped Cream",
+          "description": null,
+          "sizes": {},
+          "price": 1.40,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Super Waffle Combo",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Waffle Combo",
+          "description": "Waffle combo with Two Eggs* with choice of Bacon, or Sausage Patties, or Liver Mush or Beef Bologna and Grits, or Hash Browns or Home Fries.",
+          "sizes": {},
+          "price": 11.45,
+          "modifierGroup": null,
+          "itemType": "combo",
+          "comboGroups": [
+            {
+              "groupName": "Waffle",
+              "isInclude": true,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Waffle", "price": 0 }
+              ]
+            },
+            {
+              "groupName": "Eggs",
+              "isInclude": true,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Two Eggs", "price": 0 }
+              ]
+            },
+            {
+              "groupName": "Choice of Meat",
+              "isInclude": false,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Bacon", "price": 0 },
+                { "name": "Sausage Patties", "price": 0 },
+                { "name": "Liver Mush", "price": 0 },
+                { "name": "Beef Bologna", "price": 0 }
+              ]
+            },
+            {
+              "groupName": "Choice of Side",
+              "isInclude": false,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Grits", "price": 0 },
+                { "name": "Hash Browns", "price": 0 },
+                { "name": "Home Fries", "price": 0 }
+              ]
+            }
+          ]
+        }
+      ]
+    },
+    {
+      "category": "Juices",
+      "lstInvSize": true,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Orange",
+          "description": null,
+          "sizes": { "Small": 2.95, "Large": 3.45 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Apple",
+          "description": null,
+          "sizes": { "Small": 2.95, "Large": 3.45 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Cranberry",
+          "description": null,
+          "sizes": { "Small": 2.95, "Large": 3.45 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Beverages",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Soft Drinks",
+          "description": null,
+          "sizes": {},
+          "price": 2.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Iced Tea",
+          "description": null,
+          "sizes": {},
+          "price": 2.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Coffee",
+          "description": null,
+          "sizes": {},
+          "price": 2.50,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Hot Tea",
+          "description": null,
+          "sizes": {},
+          "price": 2.50,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Hot Chocolate",
+          "description": null,
+          "sizes": {},
+          "price": 2.50,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Milk",
+          "description": null,
+          "sizes": { "Sm": 2.25, "Lrg": 2.95 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Chocolate Milk",
+          "description": null,
+          "sizes": { "Sm": 2.25, "Lrg": 2.95 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    }
+  ],
+  "modifierGroups": [
+    {
+      "groupName": "Omelettes Serving Choice",
+      "type": "modifier",
+      "lstInvSize": false,
+      "options": [
+        {
+          "name": "Choose Side",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": "Choose Side Options"
+        },
+        {
+          "name": "Choose Bread",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": "Choose Bread Options"
+        }
+      ]
+    },
+    {
+      "groupName": "Choose Side Options",
+      "type": "modifier",
+      "lstInvSize": false,
+      "options": [
+        {
+          "name": "Hash Browns",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Grits",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Home Fries",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        }
+      ]
+    },
+    {
+      "groupName": "Choose Bread Options",
+      "type": "modifier",
+      "lstInvSize": false,
+      "options": [
+        {
+          "name": "Toast",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Biscuit",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        }
+      ]
+    },
+    {
+      "groupName": "Waffle Meat Modifiers",
+      "type": "modifier",
+      "lstInvSize": false,
+      "options": [
+        {
+          "name": "Bacon",
+          "price": 8.95,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Sausage Patties",
+          "price": 8.95,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Bologna",
+          "price": 8.95,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Liver Mush",
+          "price": 8.95,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Ham",
+          "price": 9.25,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Links",
+          "price": 9.25,
+          "prices": {},
+          "modifierGroup": null
+        }
+      ]
+    }
+  ]
+}
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-17T12:02:37.580881+00:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>menu_api_call</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>arn:aws:bedrock:us-east-1:078805859846:inference-profile/us.anthropic.claude-sonnet-4-6</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>9056</v>
+      </c>
+      <c r="E22" t="n">
+        <v>5680</v>
+      </c>
+      <c r="F22" t="n">
+        <v>14736</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You are a structured data extraction engine.
+Task:
+Extract menu information from the provided menu image and convert it into structured JSON.
+Follow all rules strictly.
+--------------------------------------------------
+1. CATEGORY GROUPING
+--------------------------------------------------
+- Group all items under their respective category names.
+- Do not merge categories.
+- Do not skip any item.
+--------------------------------------------------
+2. SIZE HANDLING (Category-Level Sizes)
+--------------------------------------------------
+If a category contains size columns like R, M, L (or Small/Medium/Large or sml/lrg/Half/Full):
+    "lstInvSize": true
+Each item must use:
+    "sizes": { "R": price, "M": price, "L": price }
+    (use whatever size keys appear in the menu header, e.g. "S"/"M"/"L", "Half"/"Full", "sml"/"lrg")
+If a specific item in an R/M/L category is only available in one size (e.g. only M is priced):
+    Include only that size key in "sizes": { "M": price }
+    Do NOT force all size keys if they are blank or missing for that item.
+If a category has only one fixed size labeled "Only Medium" or similar:
+    "lstInvSize": false
+    "sizeType": "ONLY_MEDIUM"
+Use:
+    "price": value
+If a category has text-based size in the price itself (e.g. "sml 5.99/lrg 9.99"):
+    Treat as lstInvSize: true and extract the key-value pairs as sizes.
+If no size exists at all:
+    "lstInvSize": false
+    "sizeType": null
+--------------------------------------------------
+2B. MIXED SIZE CATEGORIES (PER-ITEM SIZES)
+--------------------------------------------------
+Some categories are otherwise flat, single-price categories, but ONE or A FEW individual items show their own inline size-based pricing directly in that item's row (e.g. "Milk Sm 2.25 ... Lrg 2.95" inside a category where every other item has one plain price).
+In this case:
+- Do NOT apply sizes to the whole category.
+- Leave the category as flat ("lstInvSize": false, "sizeType": null) if most items are plain-priced.
+- For the specific item(s) that show inline sizes, set:
+    "sizes": { "Sm": price, "Lrg": price }
+    (use whatever size labels appear next to that item, e.g. "Sm"/"Lrg", "Small"/"Large", "Half"/"Full")
+    "price": null
+- All other items in that category keep their normal single "price" value and empty "sizes": {}.
+Example:
+  Category "Beverages" (flat, single price):
+    - "Coffee"       → "price": 2.50, "sizes": {}
+    - "Milk"         → "price": null, "sizes": { "Sm": 2.25, "Lrg": 2.95 }
+--------------------------------------------------
+2C. PORTION-SIZE TIERS SHARING ONE DESCRIPTION (AVOID DUPLICATE ITEMS)
+--------------------------------------------------
+Some menus present ONE dish/description followed by several named portion-size tiers with different prices — shown as boxes, a header table, or inline labels (e.g. MINI/SENIOR/REGULAR/XLARGE, Small/Medium/Large/Family, Personal/Regular/Large, 4pcs/7pcs/12pcs/20pcs, Half/Full). This can happen regardless of visual layout — boxes, a table, or plain inline text — not just an inline R/M/L column next to the item row.
+DETECTION RULE (works for ANY menu style, ANY tier wording):
+Before finalizing items in a category, check: are you about to create MORE THAN ONE item that share the EXACT SAME (or near-identical) name/description and differ ONLY by a size/portion/quantity label and its price? If yes, STOP — merge them into ONE item instead.
+Rule:
+- Create exactly ONE item using the shared description.
+- "sizes": { "&lt;tier label 1&gt;": price, "&lt;tier label 2&gt;": price, ... } — use the exact tier labels/wording printed on the menu (e.g. "Mini", "Senior", "Regular", "XLarge", "4pcs", "7pcs").
+- "price": null (the price lives entirely in "sizes").
+- Do NOT create a separate item per tier, even if the tiers are printed in separate boxes/columns/callouts rather than a single row.
+This generalizes Section 2 to portion/quantity-tier wording beyond R/M/L, and applies to any category where one dish is offered at multiple named tiers.
+--------------------------------------------------
+3. PRICE FORMAT DETECTION
+--------------------------------------------------
+Before mapping prices to items or modifier options, parse prices using these rules:
+A) Single numeric price:
+   "120/-"   → 120
+   "120"     → 120
+   "$5.99"   → 5.99
+B) Two prices separated by "/" or " " (slash/space):
+   "140/- 160/-"   → [140, 160]
+   "140/160"       → [140, 160]
+   "5.99/lrg 9.99" → handled as sizes (see Section 2)
+C) Three or more prices — concatenated with "/-" or "/" or space:
+   "150/-160/-170/-"    → [150, 160, 170]
+   "150/160/170"        → [150, 160, 170]
+   "200/-220/-210/-"    → [200, 220, 210]
+D) Multi-line prices (prices split across two visual lines in the menu):
+   Concatenate all price tokens for that item row and map sequentially.
+   Example: first line "150/-160/-170/-", second line "170/-160/-"
+   → combined prices: [150, 160, 170, 170, 160]
+E) "MRP" price (no fixed price printed):
+   "price": null
+F) If price count and modifier option count mismatch:
+   Map sequentially. Assign 0 to any remaining options without a price.
+--------------------------------------------------
+4. ITEM-LEVEL MODIFIER DETECTION
+--------------------------------------------------
+If an item name contains option patterns such as:
+- (Veg/Non Veg)
+- (Veg / Non Veg)
+- (Paneer, Baby Corn, Mushroom, Gobi)
+- (Chicken, Prawn, Fish)
+- Any slash-separated or comma-separated values inside brackets
+Then treat this as ITEM-LEVEL MODIFIER.
+EXCEPTION — Single-label items: If the bracket contains only ONE value like "(Non Veg)" or "(Veg)" and the item has a single price, do NOT create a modifier. Simply strip the bracket and use the item name as-is with that single price.
+For all other bracket patterns, You MUST:
+A) Set category:
+   "lstInventoryModifiers": true
+B) Remove bracket content from item name.
+C) Create a separate modifier group per item:
+{
+  "groupName": "Item Name Modifiers",
+  "type": "modifier",
+  "lstInvSize": false,
+  "options": [
+    {
+      "name": "Option Name",
+      "price": 0,
+      "modifierGroup": null
+    }
+  ]
+}
+D) Price Mapping Rules (use Section 3 to parse prices first):
+Parse all prices from the item's price field, then map sequentially:
+   First price  → First modifier option
+   Second price → Second modifier option
+   Third price  → Third modifier option
+   ...and so on.
+If more options than prices: assign price 0 to remaining options.
+If more prices than options: map sequentially, ignore extras.
+E) Item structure when modifier exists:
+{
+  "name": "Item Name",
+  "description": null,
+  "sizes": {},
+  "price": null,
+  "modifierGroup": "Item Name Modifiers"
+}
+IMPORTANT:
+- Do NOT keep combined price at item level.
+- Move all pricing into modifier options.
+- EXCEPTION: if every option costs the SAME amount (i.e. the menu prints only ONE overall price and the choice doesn't change it), do NOT null the item price — see Section 4C instead.
+--------------------------------------------------
+4B. TEXTUAL CHOICE MODIFIER (NO BRACKETS)
+--------------------------------------------------
+Some items offer a choice between named options WITHOUT brackets, expressed as plain text such as:
+   "with Bacon, or Sausage Patties, or Bologna, or Liver Mush ... 8.95"
+   "with Ham or Links ... 9.25"
+   "choice of A, or B ... price"
+If an item's text lists two or more named choices (separated by commas and/or "or") introduced by words like "with" / "choice of" / "your choice of", AND different choice groups carry DIFFERENT prices (multi-tier pricing for the same base item), treat this as an ITEM-LEVEL MODIFIER using the same structure as Section 4:
+A) Set category: "lstInventoryModifiers": true
+B) Strip the choice text from the item name, keeping only the base item name (e.g. "Waffle").
+C) Create ONE modifier group for the item:
+{
+  "groupName": "Item Name Modifiers",
+  "type": "modifier",
+  "lstInvSize": false,
+  "options": [
+    { "name": "Choice A", "price": 0, "modifierGroup": null },
+    { "name": "Choice B", "price": 0, "modifierGroup": null }
+  ]
+}
+D) Split EACH individual choice name (comma/"or"-separated) within a price tier into its OWN modifier option, and assign that tier's price to every option within that tier.
+   Example: "with Bacon, or Sausage Patties, or Bologna, or Liver Mush ... 8.95 with Ham or Links ... 9.25"
+   → options: Bacon (8.95), Sausage Patties (8.95), Bologna (8.95), Liver Mush (8.95), Ham (9.25), Links (9.25)
+E) Item structure when this modifier exists:
+{
+  "name": "Waffle",
+  "description": null,
+  "sizes": {},
+  "price": null,
+  "modifierGroup": "Waffle Modifiers"
+}
+F) Do NOT trigger this rule (the multi-tier price split) for plain descriptive "choice of" text that has only ONE price for the whole item. Only trigger THIS rule (4B) when different choice groups map to DIFFERENT prices. When there is only ONE overall price, still capture the choice as a modifier — without splitting the price — per Section 4D.
+--------------------------------------------------
+4C. PRICE RETENTION RULE FOR NO-COST CHOICE MODIFIERS
+--------------------------------------------------
+Before nulling an item's "price" because a modifier group exists (Sections 4, 4B, 6, 7), check whether the modifier's options actually change the total price:
+- If EVERY option in the modifier group costs the SAME amount (including all being 0) — meaning the choice is just a variant/flavor/filling pick and the menu prints only ONE overall price for the item — then:
+    - KEEP the item's own "price" as that single printed price (do NOT null it).
+    - Set every option's "price" to 0 (the cost is already included in the item price).
+- Only set the item's "price" to null when different options carry genuinely DIFFERENT prices that change what the customer pays (a true upcharge/price-tier modifier, as in Section 4B).
+This rule applies globally to item-level (4/4B), category-level (6), and shared category-level (7) modifiers — never lose the printed price of an item just because it also offers a same-price choice.
+Example: "Pie Special — ALL £11.75 — Choose from: Steak, Meat &amp; Potato, Cheese &amp; Onion, Meat Pie, Steak Pudding" → "price": 11.75 (kept), every filling option priced 0.
+--------------------------------------------------
+4D. SINGLE-PRICE CHOICE MODIFIER (FLAT ALTERNATIVES, NO PRICE SPLIT)
+--------------------------------------------------
+Some items or categories list several named alternatives (flavors, fillings, proteins, sauces, toppings, etc. — separated by commas/"or"/newlines) where the menu prints only ONE overall price (no per-choice price difference). Examples: "Pie Special — ALL £11.75 — Choose from: Steak, Meat &amp; Potato, Cheese &amp; Onion, Meat Pie, Steak Pudding" or "Crispy Shredded Chicken — Choose a flavour! Plain, Salt &amp; Pepper or Salt &amp; Chilli — £11.75".
+For this pattern:
+A) Keep the item's own "price" as the single printed price (per Section 4C — do NOT null it).
+B) Still capture every named alternative as a modifier — do NOT drop the choice information just because there's no price split. Wrap ALL alternatives under ONE modifier group named after what is being chosen (e.g. "Choice of Filling", "Choice of Flavour"), using the NESTED MODIFIER GROUP mechanism from Section 8:
+   - The item's (or category's) own modifierGroup has exactly ONE option — the wrapping choice name (e.g. "Choice of Filling") — whose own "modifierGroup" field points to a second modifierGroups entry.
+   - That second modifierGroups entry lists every named alternative (Steak, Meat &amp; Potato, Cheese &amp; Onion, ...) as its options, each "price": 0.
+C) Do NOT create one separate top-level modifier per alternative (e.g. do NOT create 5 separate sibling groups named "Steak", "Meat &amp; Potato", etc. each with no sub-options) — every alternative must be a nested option inside the ONE wrapping group.
+D) This applies whether the choice is described at item level (Section 4) or for an entire category (Section 6) — use the same item/category "modifierGroup" assignment mechanics already defined in those sections, just wrap the flat list per this rule instead of exploding it.
+--------------------------------------------------
+5. MIXED MODIFIER CATEGORIES
+--------------------------------------------------
+If a category has SOME items with bracket modifiers and SOME items without:
+- Apply item-level modifiers ONLY to items that have bracket patterns.
+- Items without brackets remain as plain items with a direct price.
+- Set category: "lstInventoryModifiers": true (because at least one item has a modifier).
+Example:
+  - "Veg Noodle" with price 120 → plain item, no modifier
+  - "Mix Noodle (Veg/Non Veg)" with prices 140/160 → item-level modifier
+--------------------------------------------------
+6. CATEGORY-LEVEL MODIFIER DETECTION
+--------------------------------------------------
+If a modifier section applies to ALL items within a single category
+(e.g., Half/Full, Regular/Large, Veg/Non Veg for whole category),
+Then:
+A) Set:
+   "lstInventoryModifiers": true
+B) Create ONE modifier group for that category:
+{
+  "groupName": "Category Name Modifiers",
+  "type": "modifier",
+  "lstInvSize": false,
+  "options": [
+    {
+      "name": "Option Name",
+      "price": 0,
+      "modifierGroup": null
+    }
+  ]
+}
+C) Assign:
+   "modifierGroup": "Category Name Modifiers"
+D) Map prices sequentially per item if multiple prices exist.
+E) Do NOT create separate modifier groups per item.
+--------------------------------------------------
+6B. CATEGORY-WIDE INCLUDED SERVING NOTE (NO PRICE, MULTIPLE CHOICE GROUPS)
+--------------------------------------------------
+Some categories carry a shared note — a header or footer line positioned ABOVE/BELOW the item list rather than inside any single item's own row/price cell — describing what EVERY item in that category is served with. Examples:
+   "Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit."
+   "Two Eggs* served with Home Fries or Grits or Hash Browns, and Toast or Biscuit."
+Treat this as a CATEGORY-LEVEL MODIFIER (Section 6) with these specifics:
+A) No price change: the note is already included in every item's own price. Follow the price-retention rule (Section 4C) — keep each item's own printed "price", and price every modifier option 0.
+B) The note may describe MORE THAN ONE independent choice group joined by "and"/commas (e.g. a side choice AND a separate bread choice). Do NOT flatten these into one list. Create ONE modifier group per distinct choice category (e.g. "Choose Side", "Choose Bread"), each wrapped using the SAME nested-wrap mechanism as Section 4D:
+   - The category's own "modifierGroup" points to ONE modifierGroups entry whose "options" are the wrapping choice names ("Choose Side", "Choose Bread", etc.), each option's own "modifierGroup" pointing to a further modifierGroups entry holding the actual named choices (e.g. Hash Browns/Grits/Home Fries under "Choose Side"; Toast/Biscuit under "Choose Bread").
+C) Apply this "modifierGroup" at the CATEGORY level (per Section 6) so it covers EVERY item in the category — do not attach it per item.
+D) Copy the shared note text into EACH item's own "description" field as well (combine with any item-specific description text if present), so no item is left with a blank description just because its serving note lives outside the item row.
+E) If the identical (or near-identical) shared note/choice set recurs across MULTIPLE categories (e.g. the same Hash Browns/Grits/Home Fries + Toast/Biscuit choice appears under an omelette category, a steak-and-eggs category, and a fish category), do NOT rebuild duplicate modifier groups per category. Define the wrapping group and its nested choice groups ONCE in "modifierGroups", and assign that SAME "modifierGroup" name to every matching category — this qualifies as a SHARED CATEGORY-LEVEL MODIFIER (Section 7) even without an explicitly named header like "Extra Topping."
+F) This pattern is not limited to breakfast sides — any cuisine/menu style where a whole category shares an included, no-extra-cost choice note (e.g. "Served with rice or naan", "Includes soup or salad", "Comes with fries or side salad") follows this same rule.
+--------------------------------------------------
+7. SHARED CATEGORY-LEVEL MODIFIER (MULTIPLE CATEGORIES)
+--------------------------------------------------
+If a separate section exists such as:
+- Extra Topping
+- Add Ons
+- Upgrade Options
+- Additional Toppings
+...OR a repeated shared serving note without a distinct named header (see Section 6B-E, e.g. the same "served with X or Y" choice printed under several categories)
+And it clearly applies to multiple categories
+(e.g., American Veg Pizza, Desi Veg Pizza, Italian Veg Pizza),
+Then treat it as SHARED CATEGORY-LEVEL MODIFIER.
+You MUST:
+A) Create ONE shared modifier group:
+{
+  "groupName": "Extra Topping",
+  "type": "modifier",
+  "lstInvSize": true/false,
+  "options": [
+    {
+      "name": "Extra Cheese",
+      "price": 0,
+      "prices": { "R": 40, "M": 60, "L": 90 },
+      "modifierGroup": null
+    }
+  ]
+}
+B) If modifier pricing depends on size (R/M/L):
+   "lstInvSize": true
+   Use:
+      "prices": { "R": value, "M": value, "L": value }
+C) If single price:
+   "lstInvSize": false
+   Use: "price": value
+D) Assign this modifier group to ALL applicable categories:
+{
+  "category": "American Veg Pizza",
+  "lstInventoryModifiers": true,
+  "modifierGroup": "Extra Topping"
+}
+E) Do NOT duplicate shared modifier groups.
+--------------------------------------------------
+8. NESTED MODIFIER GROUP (MODIFIER INSIDE MODIFIER)
+--------------------------------------------------
+If a modifier option itself contains selectable options visible in the menu
+(example: Extra Cheese → shows sub-list: Mozzarella, Cheddar, Parmesan)
+Then treat this as a NESTED MODIFIER GROUP.
+You MUST:
+A) Create a separate modifier group for the inner modifier:
+{
+  "groupName": "Extra Cheese Type",
+  "type": "modifier",
+  "lstInvSize": false,
+  "options": [
+    {
+      "name": "Mozzarella",
+      "price": 0,
+      "modifierGroup": null
+    },
+    {
+      "name": "Cheddar",
+      "price": 0,
+      "modifierGroup": null
+    }
+  ]
+}
+B) Attach this nested group to the parent modifier option:
+{
+  "name": "Extra Cheese",
+  "price": 40,
+  "modifierGroup": "Extra Cheese Type"
+}
+C) Nested modifier must NOT duplicate pricing unless explicitly shown.
+D) Nested modifiers can exist under:
+   Item-level modifier
+   Category-level modifier
+   Shared category-level modifier
+E) Maintain hierarchy strictly:
+   Category → Item → Modifier → Nested Modifier
+--------------------------------------------------
+9. ITEMS WITHOUT MODIFIERS
+--------------------------------------------------
+If item has:
+- No size
+- No modifier
+- No variation
+Then:
+{
+  "name": "",
+  "description": null,
+  "sizes": {},
+  "price": value,
+  "modifierGroup": null
+}
+If price is MRP (no fixed price printed):
+  "price": null
+And category:
+    "lstInventoryModifiers": false
+--------------------------------------------------
+9B. ITEM TYPE DETECTION (PRODUCT VS COMBO)
+--------------------------------------------------
+Every item must be classified with an "itemType" field:
+- Set "itemType": "combo" if:
+    - The item name or its category name contains bundle wording such as "Combo", "Meal", "Set Meal", "Value Meal", "Platter Combo", or similar, OR
+    - The item explicitly bundles multiple separate components into one fixed price (e.g. "Waffle Combo w/ Two Eggs, Bacon or Sausage, and Toast").
+- Otherwise set "itemType": "product" (default for all normal, non-bundled menu items).
+For "itemType": "combo" items:
+   - Do NOT use "modifierGroup" / "sizes" for the combo's bundled components — use "comboGroups" instead (see Section 9C).
+   - "sizes" stays {} and "modifierGroup" stays null on the item, unless the combo itself is separately offered in multiple sizes.
+   - "price" is the combo's own total price (e.g. 11.45).
+For "itemType": "product" items, "comboGroups" stays [] (unused) and normal "sizes" / "modifierGroup" rules (Sections 2, 2B, 4, 4B, 6, 7) apply as usual.
+CONSISTENCY RULE: If the exact same item name/description text appears in more than one category/section of the menu (e.g. the same combo listed both in a "Combos" section and again in a "Mains" section), classify and structure it IDENTICALLY everywhere it appears — same "itemType", same "sizes"/"comboGroups"/"modifierGroup" breakdown, same level of detail. Base classification purely on the item's own text — never on which category box or section it happens to be printed in.
+--------------------------------------------------
+9C. COMBO COMPONENT BREAKDOWN ("comboGroups")
+--------------------------------------------------
+For every "itemType": "combo" item, break down its bundled components into "comboGroups". Read the combo's full text (e.g. "Two Eggs* with choice of Bacon, Sausage Patties, Liver Mush or Beef Bologna, served with Grits, Hash Browns, or Home Fries, and a Waffle") and identify each distinct component:
+A) FIXED / INCLUDED component (no choice, always part of the combo, e.g. "Two Eggs", "a Waffle", "Toast or Biscuit" if only one is always given):
+   - One comboGroup per fixed component.
+   - "isInclude": true
+   - "minQty": 1, "maxQty": 1
+   - Exactly ONE option in "options", price 0 (already covered by the combo price) unless the menu prints an explicit extra charge.
+B) CHOICE component (customer selects one from a named list, e.g. "choice of Bacon, Sausage Patties, Liver Mush or Beef Bologna"):
+   - One comboGroup per distinct choice category (e.g. "Choice of Meat", "Choice of Side", "Choice of Bread").
+   - "isInclude": false
+   - "minQty": 1, "maxQty": 1 (or higher "maxQty" only if the menu explicitly allows selecting more than one)
+   - Split each named choice (comma/"or"-separated) into its own option, price 0 unless the menu shows an explicit add-on charge for that specific choice.
+C) Name each comboGroup by what it represents (e.g. "Eggs", "Choice of Meat", "Choice of Side"), not generically.
+D) Combine the combo's full bundled text into one natural-language sentence in the item's "description" field (e.g. "Two eggs with choice of bacon, sausage patties, liver mush or beef bologna, served with grits, hash browns, or home fries and a waffle.").
+E) Structure:
+{
+  "name": "Super Waffle Combo",
+  "description": "Two eggs with choice of bacon, sausage patties, liver mush or beef bologna, served with grits or hash browns or home fries and a waffle combo.",
+  "sizes": {},
+  "price": 11.45,
+  "modifierGroup": null,
+  "itemType": "combo",
+  "comboGroups": [
+    {
+      "groupName": "Eggs",
+      "isInclude": true,
+      "minQty": 1,
+      "maxQty": 1,
+      "options": [ { "name": "Two Eggs", "price": 0 } ]
+    },
+    {
+      "groupName": "Choice of Meat",
+      "isInclude": false,
+      "minQty": 1,
+      "maxQty": 1,
+      "options": [
+        { "name": "Bacon", "price": 0 },
+        { "name": "Sausage Patties", "price": 0 },
+        { "name": "Liver Mush", "price": 0 },
+        { "name": "Beef Bologna", "price": 0 }
+      ]
+    },
+    {
+      "groupName": "Choice of Side",
+      "isInclude": false,
+      "minQty": 1,
+      "maxQty": 1,
+      "options": [
+        { "name": "Grits", "price": 0 },
+        { "name": "Hash Browns", "price": 0 },
+        { "name": "Home Fries", "price": 0 }
+      ]
+    }
+  ]
+}
+F) This applies to ANY combo menu, not just breakfast combos — pizza combos, burger combos, thali/set-meal combos, etc. Always decompose into "fixed inclusion" groups vs "choice" groups using rules A and B above, regardless of cuisine or category name.
+--------------------------------------------------
+10. MODIFIER PRIORITY RULE
+--------------------------------------------------
+1. If modifier applies only to one item → Item-Level Modifier.
+2. If modifier applies to entire category → Category-Level Modifier.
+3. If modifier applies to multiple categories → Shared Category-Level Modifier.
+4. If modifier option has sub-options → Nested Modifier Group.
+5. Never duplicate modifier groups.
+--------------------------------------------------
+11. FINAL STRUCTURE (STRICT FORMAT)
+--------------------------------------------------
+Return ONLY this JSON structure:
+{
+  "categories": [
+    {
+      "category": "",
+      "lstInvSize": true/false,
+      "lstInventoryModifiers": true/false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "",
+          "description": null,
+          "sizes": {},
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    }
+  ],
+  "modifierGroups": [
+    {
+      "groupName": "",
+      "type": "modifier",
+      "lstInvSize": true/false,
+      "options": [
+        {
+          "name": "",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        }
+      ]
+    }
+  ]
+}
+--------------------------------------------------
+12. STRICT RULES
+--------------------------------------------------
+- Do not skip any item.
+- Keep prices as numbers only (no "/- " suffix, no currency symbols).
+- Remove brackets and their content from item names.
+- Do not duplicate modifier groups.
+- Do not leave price at item level if a modifier group exists, UNLESS every option in that modifier group is equal-price/no-cost (see Section 4C) — in that case keep the item price and set option prices to 0.
+- If price count and modifier count mismatch, map sequentially; assign 0 to unpaired options.
+- Nested modifiers must reference parent modifier correctly.
+- If a field is not applicable, set it to null (NOT empty string "").
+- "sizeType" must be null unless it is "ONLY_MEDIUM".
+- "modifierGroup" at category or item level must be null when not applicable.
+- "prices" field in modifier options must be {} (empty object) when not applicable.
+- "itemType" must be "product" for every regular item, and "combo" only for bundled/combo items (see Section 9B).
+- "comboGroups" must be [] for "product" items, and fully populated (fixed + choice groups, see Section 9C) for "combo" items.
+- Do not create multiple items in a category that share the same name/description and differ only by a size/portion tier label — merge into one item with "sizes" instead (see Section 2C).
+- If the same item text appears in more than one category, classify and structure it identically everywhere (see Section 9B consistency rule).
+- Do not leave "description" blank or skip modifiers just because a category's serving note (e.g. "served with X or Y, and A or B") sits outside the item row — apply it to every item in the category per Section 6B.
+- Return ONLY valid JSON.
+- Do NOT add explanations.
+- Do NOT use markdown.
+- Do not miss any itam details recheck and found any things is missing add the item proper as per rule
+</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>```json
+{
+  "categories": [
+    {
+      "category": "American Veg Pizza",
+      "lstInvSize": true,
+      "lstInventoryModifiers": true,
+      "sizeType": null,
+      "modifierGroup": "Extra Topping",
+      "items": [
+        {
+          "name": "Margherita Pizza",
+          "description": "Lots of Cheese",
+          "sizes": { "R": 125, "M": 275, "L": 400 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Vegetarian Bite",
+          "description": "Cheese, green pepper, tomato, onions",
+          "sizes": { "R": 165, "M": 315, "L": 500 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Mushroom Riot",
+          "description": "Cheese, mushroom, garlic, chilli",
+          "sizes": { "R": 275, "M": 335, "L": 525 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Mexican Delight",
+          "description": "Cheese, chilly, sweet corn, tomato, olives",
+          "sizes": { "R": 245, "M": 360, "L": 545 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "American Heat",
+          "description": "Cheese, green pepper, onion, baby corn, jalapeno",
+          "sizes": { "R": 245, "M": 360, "L": 545 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Spicy Treat",
+          "description": "Cheese, green pepper, spicy paneer, olives, jalapeno",
+          "sizes": { "R": 245, "M": 360, "L": 545 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Hawaiian Fantasy",
+          "description": "Cheese, mushroom, pineapple, BBQ Paneer jalapeno",
+          "sizes": { "R": 265, "M": 420, "L": 570 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Fresh Veggi Special",
+          "description": "Cheese, onion, green pepper, mushroom, tomato, olives, sweet corn, paneer",
+          "sizes": { "R": 265, "M": 420, "L": 570 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Cheese Burst",
+          "description": "3 kind of cheese, onion, capsicum, paneer &amp; Jalapeno",
+          "sizes": { "M": 333 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Desi Veg Pizza",
+      "lstInvSize": true,
+      "lstInventoryModifiers": true,
+      "sizeType": null,
+      "modifierGroup": "Extra Topping",
+      "items": [
+        {
+          "name": "Tandoori Paneer",
+          "description": "Cheese, onion, Green pepper, Tomato, Coriander, Tandoori paneer, makhni sprinkle",
+          "sizes": { "R": 225, "M": 335, "L": 525 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Yum Dum",
+          "description": "Cheese, Onion, Spinach, Spicy Paneer, Chilly, Garlic, makhni sprinkle",
+          "sizes": { "R": 245, "M": 360, "L": 545 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Balle Balle",
+          "description": "Cheese, onion, tandoori paneer, chilly, coriander, makhani sprinkle",
+          "sizes": { "R": 245, "M": 360, "L": 545 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Gujarati Treat",
+          "description": "Cheese, onion, green pepper, chilly, garlic, green pea masala, tomato, coriander",
+          "sizes": { "R": 265, "M": 420, "L": 570 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Chatpatta Paneer",
+          "description": "Cheese, sweet corn, chatpatta paneer, tomato, coriander, chettinad sprinkle",
+          "sizes": { "R": 265, "M": 420, "L": 570 },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Pav Bhaji",
+          "description": "Cheese, pavbhaji mix, butter, onion, tomato &amp; coriander",
+          "sizes": {},
+          "price": 299,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Italian Veg Pizza",
+      "lstInvSize": false,
+      "lstInventoryModifiers": true,
+      "sizeType": "ONLY_MEDIUM",
+      "modifierGroup": "Extra Topping",
+      "items": [
+        {
+          "name": "Classic Margherita",
+          "description": "Rustica tomato, Basil &amp; mozarella",
+          "sizes": {},
+          "price": 250,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Funghi De Bosco",
+          "description": "Mushrooms, garlic oil, basil, Jalapenos &amp; mozarella",
+          "sizes": {},
+          "price": 350,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Giardinera",
+          "description": "Mixed peppers, santos tomatoes, Olives, Mushrooms &amp; cheese",
+          "sizes": {},
+          "price": 280,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Char Grilled",
+          "description": "Green &amp; yellow zucchini, mixed peppers, rustica tomatoes, paprika with mozarella",
+          "sizes": {},
+          "price": 280,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Quattro Formaggie",
+          "description": "Mozarella, cheddar, parmesean &amp; Cream cheese",
+          "sizes": {},
+          "price": 350,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Breads",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Garlic Bread",
+          "description": null,
+          "sizes": {},
+          "price": 75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Garlic Bread 'N' Cheese",
+          "description": null,
+          "sizes": {},
+          "price": 115,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Supreme Garlic Bread",
+          "description": null,
+          "sizes": {},
+          "price": 125,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Jain Bread",
+          "description": null,
+          "sizes": {},
+          "price": 75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Jain Bread 'N' Cheese",
+          "description": null,
+          "sizes": {},
+          "price": 115,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Supreme Jain Bread",
+          "description": null,
+          "sizes": {},
+          "price": 125,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Stuffed Garlic Bread",
+          "description": null,
+          "sizes": {},
+          "price": 125,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Starter",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Potato Wedges",
+          "description": null,
+          "sizes": {},
+          "price": 90,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Cheesy Potato Pops",
+          "description": null,
+          "sizes": {},
+          "price": 90,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Fresh Dough Bites",
+          "description": "Cheese, Pesto, Garlic",
+          "sizes": {},
+          "price": 90,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Signature French Fries",
+          "description": "Choice of sauces: Cream cheese, Peanut butter, Korean Bbq",
+          "sizes": {},
+          "price": 120,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Salad",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Greek Salad",
+          "description": null,
+          "sizes": {},
+          "price": 120,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Hawaiin Salad",
+          "description": null,
+          "sizes": {},
+          "price": 120,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Russian Salad",
+          "description": null,
+          "sizes": {},
+          "price": 120,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Mix Salad Bowl Veg",
+          "description": null,
+          "sizes": {},
+          "price": 120,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Wrap",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Veg Wrap",
+          "description": null,
+          "sizes": {},
+          "price": 99,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Pasta",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Roman Pasta",
+          "description": null,
+          "sizes": {},
+          "price": 120,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Creamy Indian Pasta",
+          "description": null,
+          "sizes": {},
+          "price": 120,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Pasta Alfredo",
+          "description": null,
+          "sizes": {},
+          "price": 120,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Dessert",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Brownie",
+          "description": null,
+          "sizes": {},
+          "price": 90,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Chocolate Pizza",
+          "description": null,
+          "sizes": {},
+          "price": 120,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Beverages",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Coke",
+          "description": null,
+          "sizes": {},
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Fanta",
+          "description": null,
+          "sizes": {},
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Sprite",
+          "description": null,
+          "sizes": {},
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Mineral Water",
+          "description": null,
+          "sizes": {},
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    }
+  ],
+  "modifierGroups": [
+    {
+      "groupName": "Extra Topping",
+      "type": "modifier",
+      "lstInvSize": true,
+      "options": [
+        {
+          "name": "Extra Cheese",
+          "price": 0,
+          "prices": { "R": 40, "M": 60, "L": 90 },
+          "modifierGroup": "Extra Cheese Type"
+        },
+        {
+          "name": "Choice of Sauces",
+          "price": 0,
+          "prices": { "R": 20, "M": 40, "L": 60 },
+          "modifierGroup": "Choice of Sauces Type"
+        },
+        {
+          "name": "Upgrade to Thin Crust",
+          "price": 0,
+          "prices": { "R": 30, "M": 60, "L": 90 },
+          "modifierGroup": null
+        },
+        {
+          "name": "Extra Veg Topping",
+          "price": 0,
+          "prices": { "R": 25, "M": 50, "L": 75 },
+          "modifierGroup": "Extra Veg Topping Type"
+        }
+      ]
+    },
+    {
+      "groupName": "Extra Cheese Type",
+      "type": "modifier",
+      "lstInvSize": false,
+      "options": [
+        {
+          "name": "Mozzarella",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Cheddar",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Parmesan",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Cream Cheese",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        }
+      ]
+    },
+    {
+      "groupName": "Choice of Sauces Type",
+      "type": "modifier",
+      "lstInvSize": false,
+      "options": [
+        {
+          "name": "American",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Buffalo",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Desi",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Makhni",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Chipotle",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        }
+      ]
+    },
+    {
+      "groupName": "Extra Veg Topping Type",
+      "type": "modifier",
+      "lstInvSize": false,
+      "options": [
+        {
+          "name": "Onion",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Tomato",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Green Pepper",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Spinach",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Garlic Green Chilli",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Mushroom",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Green Pea Masala",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Olives",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Jalapeno",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Pineapple",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Sweet Corn",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Paneer Tandoori",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Paneer Spicy Barbeque",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Paneer Chatpata",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        }
+      ]
+    }
+  ]
+}
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07-17T12:07:11.089638+00:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>menu_api_call</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>arn:aws:bedrock:us-east-1:078805859846:inference-profile/us.anthropic.claude-sonnet-4-6</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>9089</v>
+      </c>
+      <c r="E23" t="n">
+        <v>7295</v>
+      </c>
+      <c r="F23" t="n">
+        <v>16384</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You are a structured data extraction engine.
+Task:
+Extract menu information from the provided menu image and convert it into structured JSON.
+Follow all rules strictly.
+--------------------------------------------------
+1. CATEGORY GROUPING
+--------------------------------------------------
+- Group all items under their respective category names.
+- Do not merge categories.
+- Do not skip any item.
+--------------------------------------------------
+2. SIZE HANDLING (Category-Level Sizes)
+--------------------------------------------------
+If a category contains size columns like R, M, L (or Small/Medium/Large or sml/lrg/Half/Full):
+    "lstInvSize": true
+Each item must use:
+    "sizes": { "R": price, "M": price, "L": price }
+    (use whatever size keys appear in the menu header, e.g. "S"/"M"/"L", "Half"/"Full", "sml"/"lrg")
+If a specific item in an R/M/L category is only available in one size (e.g. only M is priced):
+    Include only that size key in "sizes": { "M": price }
+    Do NOT force all size keys if they are blank or missing for that item.
+If a category has only one fixed size labeled "Only Medium" or similar:
+    "lstInvSize": false
+    "sizeType": "ONLY_MEDIUM"
+Use:
+    "price": value
+If a category has text-based size in the price itself (e.g. "sml 5.99/lrg 9.99"):
+    Treat as lstInvSize: true and extract the key-value pairs as sizes.
+If no size exists at all:
+    "lstInvSize": false
+    "sizeType": null
+--------------------------------------------------
+2B. MIXED SIZE CATEGORIES (PER-ITEM SIZES)
+--------------------------------------------------
+Some categories are otherwise flat, single-price categories, but ONE or A FEW individual items show their own inline size-based pricing directly in that item's row (e.g. "Milk Sm 2.25 ... Lrg 2.95" inside a category where every other item has one plain price).
+In this case:
+- Do NOT apply sizes to the whole category.
+- Leave the category as flat ("lstInvSize": false, "sizeType": null) if most items are plain-priced.
+- For the specific item(s) that show inline sizes, set:
+    "sizes": { "Sm": price, "Lrg": price }
+    (use whatever size labels appear next to that item, e.g. "Sm"/"Lrg", "Small"/"Large", "Half"/"Full")
+    "price": null
+- All other items in that category keep their normal single "price" value and empty "sizes": {}.
+Example:
+  Category "Beverages" (flat, single price):
+    - "Coffee"       → "price": 2.50, "sizes": {}
+    - "Milk"         → "price": null, "sizes": { "Sm": 2.25, "Lrg": 2.95 }
+--------------------------------------------------
+2C. PORTION-SIZE TIERS SHARING ONE DESCRIPTION (AVOID DUPLICATE ITEMS)
+--------------------------------------------------
+Some menus present ONE dish/description followed by several named portion-size tiers with different prices — shown as boxes, a header table, or inline labels (e.g. MINI/SENIOR/REGULAR/XLARGE, Small/Medium/Large/Family, Personal/Regular/Large, 4pcs/7pcs/12pcs/20pcs, Half/Full). This can happen regardless of visual layout — boxes, a table, or plain inline text — not just an inline R/M/L column next to the item row.
+DETECTION RULE (works for ANY menu style, ANY tier wording):
+Before finalizing items in a category, check: are you about to create MORE THAN ONE item that share the EXACT SAME (or near-identical) name/description and differ ONLY by a size/portion/quantity label and its price? If yes, STOP — merge them into ONE item instead.
+Rule:
+- Create exactly ONE item using the shared description.
+- "sizes": { "&lt;tier label 1&gt;": price, "&lt;tier label 2&gt;": price, ... } — use the exact tier labels/wording printed on the menu (e.g. "Mini", "Senior", "Regular", "XLarge", "4pcs", "7pcs").
+- "price": null (the price lives entirely in "sizes").
+- Do NOT create a separate item per tier, even if the tiers are printed in separate boxes/columns/callouts rather than a single row.
+This generalizes Section 2 to portion/quantity-tier wording beyond R/M/L, and applies to any category where one dish is offered at multiple named tiers.
+--------------------------------------------------
+3. PRICE FORMAT DETECTION
+--------------------------------------------------
+Before mapping prices to items or modifier options, parse prices using these rules:
+A) Single numeric price:
+   "120/-"   → 120
+   "120"     → 120
+   "$5.99"   → 5.99
+B) Two prices separated by "/" or " " (slash/space):
+   "140/- 160/-"   → [140, 160]
+   "140/160"       → [140, 160]
+   "5.99/lrg 9.99" → handled as sizes (see Section 2)
+C) Three or more prices — concatenated with "/-" or "/" or space:
+   "150/-160/-170/-"    → [150, 160, 170]
+   "150/160/170"        → [150, 160, 170]
+   "200/-220/-210/-"    → [200, 220, 210]
+D) Multi-line prices (prices split across two visual lines in the menu):
+   Concatenate all price tokens for that item row and map sequentially.
+   Example: first line "150/-160/-170/-", second line "170/-160/-"
+   → combined prices: [150, 160, 170, 170, 160]
+E) "MRP" price (no fixed price printed):
+   "price": null
+F) If price count and modifier option count mismatch:
+   Map sequentially. Assign 0 to any remaining options without a price.
+--------------------------------------------------
+4. ITEM-LEVEL MODIFIER DETECTION
+--------------------------------------------------
+If an item name contains option patterns such as:
+- (Veg/Non Veg)
+- (Veg / Non Veg)
+- (Paneer, Baby Corn, Mushroom, Gobi)
+- (Chicken, Prawn, Fish)
+- Any slash-separated or comma-separated values inside brackets
+Then treat this as ITEM-LEVEL MODIFIER.
+EXCEPTION — Single-label items: If the bracket contains only ONE value like "(Non Veg)" or "(Veg)" and the item has a single price, do NOT create a modifier. Simply strip the bracket and use the item name as-is with that single price.
+For all other bracket patterns, You MUST:
+A) Set category:
+   "lstInventoryModifiers": true
+B) Remove bracket content from item name.
+C) Create a separate modifier group per item:
+{
+  "groupName": "Item Name Modifiers",
+  "type": "modifier",
+  "lstInvSize": false,
+  "options": [
+    {
+      "name": "Option Name",
+      "price": 0,
+      "modifierGroup": null
+    }
+  ]
+}
+D) Price Mapping Rules (use Section 3 to parse prices first):
+Parse all prices from the item's price field, then map sequentially:
+   First price  → First modifier option
+   Second price → Second modifier option
+   Third price  → Third modifier option
+   ...and so on.
+If more options than prices: assign price 0 to remaining options.
+If more prices than options: map sequentially, ignore extras.
+E) Item structure when modifier exists:
+{
+  "name": "Item Name",
+  "description": null,
+  "sizes": {},
+  "price": null,
+  "modifierGroup": "Item Name Modifiers"
+}
+IMPORTANT:
+- Do NOT keep combined price at item level.
+- Move all pricing into modifier options.
+- EXCEPTION: if every option costs the SAME amount (i.e. the menu prints only ONE overall price and the choice doesn't change it), do NOT null the item price — see Section 4C instead.
+--------------------------------------------------
+4B. TEXTUAL CHOICE MODIFIER (NO BRACKETS)
+--------------------------------------------------
+Some items offer a choice between named options WITHOUT brackets, expressed as plain text such as:
+   "with Bacon, or Sausage Patties, or Bologna, or Liver Mush ... 8.95"
+   "with Ham or Links ... 9.25"
+   "choice of A, or B ... price"
+If an item's text lists two or more named choices (separated by commas and/or "or") introduced by words like "with" / "choice of" / "your choice of", AND different choice groups carry DIFFERENT prices (multi-tier pricing for the same base item), treat this as an ITEM-LEVEL MODIFIER using the same structure as Section 4:
+A) Set category: "lstInventoryModifiers": true
+B) Strip the choice text from the item name, keeping only the base item name (e.g. "Waffle").
+C) Create ONE modifier group for the item:
+{
+  "groupName": "Item Name Modifiers",
+  "type": "modifier",
+  "lstInvSize": false,
+  "options": [
+    { "name": "Choice A", "price": 0, "modifierGroup": null },
+    { "name": "Choice B", "price": 0, "modifierGroup": null }
+  ]
+}
+D) Split EACH individual choice name (comma/"or"-separated) within a price tier into its OWN modifier option, and assign that tier's price to every option within that tier.
+   Example: "with Bacon, or Sausage Patties, or Bologna, or Liver Mush ... 8.95 with Ham or Links ... 9.25"
+   → options: Bacon (8.95), Sausage Patties (8.95), Bologna (8.95), Liver Mush (8.95), Ham (9.25), Links (9.25)
+E) Item structure when this modifier exists:
+{
+  "name": "Waffle",
+  "description": null,
+  "sizes": {},
+  "price": null,
+  "modifierGroup": "Waffle Modifiers"
+}
+F) Do NOT trigger this rule (the multi-tier price split) for plain descriptive "choice of" text that has only ONE price for the whole item. Only trigger THIS rule (4B) when different choice groups map to DIFFERENT prices. When there is only ONE overall price, still capture the choice as a modifier — without splitting the price — per Section 4D.
+--------------------------------------------------
+4C. PRICE RETENTION RULE FOR NO-COST CHOICE MODIFIERS
+--------------------------------------------------
+Before nulling an item's "price" because a modifier group exists (Sections 4, 4B, 6, 7), check whether the modifier's options actually change the total price:
+- If EVERY option in the modifier group costs the SAME amount (including all being 0) — meaning the choice is just a variant/flavor/filling pick and the menu prints only ONE overall price for the item — then:
+    - KEEP the item's own "price" as that single printed price (do NOT null it).
+    - Set every option's "price" to 0 (the cost is already included in the item price).
+- Only set the item's "price" to null when different options carry genuinely DIFFERENT prices that change what the customer pays (a true upcharge/price-tier modifier, as in Section 4B).
+This rule applies globally to item-level (4/4B), category-level (6), and shared category-level (7) modifiers — never lose the printed price of an item just because it also offers a same-price choice.
+Example: "Pie Special — ALL £11.75 — Choose from: Steak, Meat &amp; Potato, Cheese &amp; Onion, Meat Pie, Steak Pudding" → "price": 11.75 (kept), every filling option priced 0.
+--------------------------------------------------
+4D. SINGLE-PRICE CHOICE MODIFIER (FLAT ALTERNATIVES, NO PRICE SPLIT)
+--------------------------------------------------
+Some items or categories list several named alternatives (flavors, fillings, proteins, sauces, toppings, etc. — separated by commas/"or"/newlines) where the menu prints only ONE overall price (no per-choice price difference). Examples: "Pie Special — ALL £11.75 — Choose from: Steak, Meat &amp; Potato, Cheese &amp; Onion, Meat Pie, Steak Pudding" or "Crispy Shredded Chicken — Choose a flavour! Plain, Salt &amp; Pepper or Salt &amp; Chilli — £11.75".
+For this pattern:
+A) Keep the item's own "price" as the single printed price (per Section 4C — do NOT null it).
+B) Still capture every named alternative as a modifier — do NOT drop the choice information just because there's no price split. Wrap ALL alternatives under ONE modifier group named after what is being chosen (e.g. "Choice of Filling", "Choice of Flavour"), using the NESTED MODIFIER GROUP mechanism from Section 8:
+   - The item's (or category's) own modifierGroup has exactly ONE option — the wrapping choice name (e.g. "Choice of Filling") — whose own "modifierGroup" field points to a second modifierGroups entry.
+   - That second modifierGroups entry lists every named alternative (Steak, Meat &amp; Potato, Cheese &amp; Onion, ...) as its options, each "price": 0.
+C) Do NOT create one separate top-level modifier per alternative (e.g. do NOT create 5 separate sibling groups named "Steak", "Meat &amp; Potato", etc. each with no sub-options) — every alternative must be a nested option inside the ONE wrapping group.
+D) This applies whether the choice is described at item level (Section 4) or for an entire category (Section 6) — use the same item/category "modifierGroup" assignment mechanics already defined in those sections, just wrap the flat list per this rule instead of exploding it.
+--------------------------------------------------
+5. MIXED MODIFIER CATEGORIES
+--------------------------------------------------
+If a category has SOME items with bracket modifiers and SOME items without:
+- Apply item-level modifiers ONLY to items that have bracket patterns.
+- Items without brackets remain as plain items with a direct price.
+- Set category: "lstInventoryModifiers": true (because at least one item has a modifier).
+Example:
+  - "Veg Noodle" with price 120 → plain item, no modifier
+  - "Mix Noodle (Veg/Non Veg)" with prices 140/160 → item-level modifier
+--------------------------------------------------
+6. CATEGORY-LEVEL MODIFIER DETECTION
+--------------------------------------------------
+If a modifier section applies to ALL items within a single category
+(e.g., Half/Full, Regular/Large, Veg/Non Veg for whole category),
+Then:
+A) Set:
+   "lstInventoryModifiers": true
+B) Create ONE modifier group for that category:
+{
+  "groupName": "Category Name Modifiers",
+  "type": "modifier",
+  "lstInvSize": false,
+  "options": [
+    {
+      "name": "Option Name",
+      "price": 0,
+      "modifierGroup": null
+    }
+  ]
+}
+C) Assign:
+   "modifierGroup": "Category Name Modifiers"
+D) Map prices sequentially per item if multiple prices exist.
+E) Do NOT create separate modifier groups per item.
+--------------------------------------------------
+6B. CATEGORY-WIDE INCLUDED SERVING NOTE (NO PRICE, MULTIPLE CHOICE GROUPS)
+--------------------------------------------------
+Some categories carry a shared note — a header or footer line positioned ABOVE/BELOW the item list rather than inside any single item's own row/price cell — describing what EVERY item in that category is served with. Examples:
+   "Served with Hash Browns, or Grits or Home Fries, and Toast or Biscuit."
+   "Two Eggs* served with Home Fries or Grits or Hash Browns, and Toast or Biscuit."
+Treat this as a CATEGORY-LEVEL MODIFIER (Section 6) with these specifics:
+A) No price change: the note is already included in every item's own price. Follow the price-retention rule (Section 4C) — keep each item's own printed "price", and price every modifier option 0.
+B) The note may describe MORE THAN ONE independent choice group joined by "and"/commas (e.g. a side choice AND a separate bread choice). Do NOT flatten these into one list. Create ONE modifier group per distinct choice category (e.g. "Choose Side", "Choose Bread"), each wrapped using the SAME nested-wrap mechanism as Section 4D:
+   - The category's own "modifierGroup" points to ONE modifierGroups entry whose "options" are the wrapping choice names ("Choose Side", "Choose Bread", etc.), each option's own "modifierGroup" pointing to a further modifierGroups entry holding the actual named choices (e.g. Hash Browns/Grits/Home Fries under "Choose Side"; Toast/Biscuit under "Choose Bread").
+C) Apply this "modifierGroup" at the CATEGORY level (per Section 6) so it covers EVERY item in the category — do not attach it per item.
+D) Copy the shared note text into EACH item's own "description" field as well (combine with any item-specific description text if present), so no item is left with a blank description just because its serving note lives outside the item row.
+E) If the identical (or near-identical) shared note/choice set recurs across MULTIPLE categories (e.g. the same Hash Browns/Grits/Home Fries + Toast/Biscuit choice appears under an omelette category, a steak-and-eggs category, and a fish category), do NOT rebuild duplicate modifier groups per category. Define the wrapping group and its nested choice groups ONCE in "modifierGroups", and assign that SAME "modifierGroup" name to every matching category — this qualifies as a SHARED CATEGORY-LEVEL MODIFIER (Section 7) even without an explicitly named header like "Extra Topping."
+F) This pattern is not limited to breakfast sides — any cuisine/menu style where a whole category shares an included, no-extra-cost choice note (e.g. "Served with rice or naan", "Includes soup or salad", "Comes with fries or side salad") follows this same rule.
+--------------------------------------------------
+7. SHARED CATEGORY-LEVEL MODIFIER (MULTIPLE CATEGORIES)
+--------------------------------------------------
+If a separate section exists such as:
+- Extra Topping
+- Add Ons
+- Upgrade Options
+- Additional Toppings
+...OR a repeated shared serving note without a distinct named header (see Section 6B-E, e.g. the same "served with X or Y" choice printed under several categories)
+And it clearly applies to multiple categories
+(e.g., American Veg Pizza, Desi Veg Pizza, Italian Veg Pizza),
+Then treat it as SHARED CATEGORY-LEVEL MODIFIER.
+You MUST:
+A) Create ONE shared modifier group:
+{
+  "groupName": "Extra Topping",
+  "type": "modifier",
+  "lstInvSize": true/false,
+  "options": [
+    {
+      "name": "Extra Cheese",
+      "price": 0,
+      "prices": { "R": 40, "M": 60, "L": 90 },
+      "modifierGroup": null
+    }
+  ]
+}
+B) If modifier pricing depends on size (R/M/L):
+   "lstInvSize": true
+   Use:
+      "prices": { "R": value, "M": value, "L": value }
+C) If single price:
+   "lstInvSize": false
+   Use: "price": value
+D) Assign this modifier group to ALL applicable categories:
+{
+  "category": "American Veg Pizza",
+  "lstInventoryModifiers": true,
+  "modifierGroup": "Extra Topping"
+}
+E) Do NOT duplicate shared modifier groups.
+--------------------------------------------------
+8. NESTED MODIFIER GROUP (MODIFIER INSIDE MODIFIER)
+--------------------------------------------------
+If a modifier option itself contains selectable options visible in the menu
+(example: Extra Cheese → shows sub-list: Mozzarella, Cheddar, Parmesan)
+Then treat this as a NESTED MODIFIER GROUP.
+You MUST:
+A) Create a separate modifier group for the inner modifier:
+{
+  "groupName": "Extra Cheese Type",
+  "type": "modifier",
+  "lstInvSize": false,
+  "options": [
+    {
+      "name": "Mozzarella",
+      "price": 0,
+      "modifierGroup": null
+    },
+    {
+      "name": "Cheddar",
+      "price": 0,
+      "modifierGroup": null
+    }
+  ]
+}
+B) Attach this nested group to the parent modifier option:
+{
+  "name": "Extra Cheese",
+  "price": 40,
+  "modifierGroup": "Extra Cheese Type"
+}
+C) Nested modifier must NOT duplicate pricing unless explicitly shown.
+D) Nested modifiers can exist under:
+   Item-level modifier
+   Category-level modifier
+   Shared category-level modifier
+E) Maintain hierarchy strictly:
+   Category → Item → Modifier → Nested Modifier
+--------------------------------------------------
+9. ITEMS WITHOUT MODIFIERS
+--------------------------------------------------
+If item has:
+- No size
+- No modifier
+- No variation
+Then:
+{
+  "name": "",
+  "description": null,
+  "sizes": {},
+  "price": value,
+  "modifierGroup": null
+}
+If price is MRP (no fixed price printed):
+  "price": null
+And category:
+    "lstInventoryModifiers": false
+--------------------------------------------------
+9B. ITEM TYPE DETECTION (PRODUCT VS COMBO)
+--------------------------------------------------
+Every item must be classified with an "itemType" field:
+- Set "itemType": "combo" if:
+    - The item name or its category name contains bundle wording such as "Combo", "Meal", "Set Meal", "Value Meal", "Platter Combo", or similar, OR
+    - The item explicitly bundles multiple separate components into one fixed price (e.g. "Waffle Combo w/ Two Eggs, Bacon or Sausage, and Toast").
+- Otherwise set "itemType": "product" (default for all normal, non-bundled menu items).
+For "itemType": "combo" items:
+   - Do NOT use "modifierGroup" / "sizes" for the combo's bundled components — use "comboGroups" instead (see Section 9C).
+   - "sizes" stays {} and "modifierGroup" stays null on the item, unless the combo itself is separately offered in multiple sizes.
+   - "price" is the combo's own total price (e.g. 11.45).
+For "itemType": "product" items, "comboGroups" stays [] (unused) and normal "sizes" / "modifierGroup" rules (Sections 2, 2B, 4, 4B, 6, 7) apply as usual.
+CONSISTENCY RULE: If the exact same item name/description text appears in more than one category/section of the menu (e.g. the same combo listed both in a "Combos" section and again in a "Mains" section), classify and structure it IDENTICALLY everywhere it appears — same "itemType", same "sizes"/"comboGroups"/"modifierGroup" breakdown, same level of detail. Base classification purely on the item's own text — never on which category box or section it happens to be printed in.
+--------------------------------------------------
+9C. COMBO COMPONENT BREAKDOWN ("comboGroups")
+--------------------------------------------------
+For every "itemType": "combo" item, break down its bundled components into "comboGroups". Read the combo's full text (e.g. "Two Eggs* with choice of Bacon, Sausage Patties, Liver Mush or Beef Bologna, served with Grits, Hash Browns, or Home Fries, and a Waffle") and identify each distinct component:
+A) FIXED / INCLUDED component (no choice, always part of the combo, e.g. "Two Eggs", "a Waffle", "Toast or Biscuit" if only one is always given):
+   - One comboGroup per fixed component.
+   - "isInclude": true
+   - "minQty": 1, "maxQty": 1
+   - Exactly ONE option in "options", price 0 (already covered by the combo price) unless the menu prints an explicit extra charge.
+B) CHOICE component (customer selects one from a named list, e.g. "choice of Bacon, Sausage Patties, Liver Mush or Beef Bologna"):
+   - One comboGroup per distinct choice category (e.g. "Choice of Meat", "Choice of Side", "Choice of Bread").
+   - "isInclude": false
+   - "minQty": 1, "maxQty": 1 (or higher "maxQty" only if the menu explicitly allows selecting more than one)
+   - Split each named choice (comma/"or"-separated) into its own option, price 0 unless the menu shows an explicit add-on charge for that specific choice.
+C) Name each comboGroup by what it represents (e.g. "Eggs", "Choice of Meat", "Choice of Side"), not generically.
+D) Combine the combo's full bundled text into one natural-language sentence in the item's "description" field (e.g. "Two eggs with choice of bacon, sausage patties, liver mush or beef bologna, served with grits, hash browns, or home fries and a waffle.").
+E) Structure:
+{
+  "name": "Super Waffle Combo",
+  "description": "Two eggs with choice of bacon, sausage patties, liver mush or beef bologna, served with grits or hash browns or home fries and a waffle combo.",
+  "sizes": {},
+  "price": 11.45,
+  "modifierGroup": null,
+  "itemType": "combo",
+  "comboGroups": [
+    {
+      "groupName": "Eggs",
+      "isInclude": true,
+      "minQty": 1,
+      "maxQty": 1,
+      "options": [ { "name": "Two Eggs", "price": 0 } ]
+    },
+    {
+      "groupName": "Choice of Meat",
+      "isInclude": false,
+      "minQty": 1,
+      "maxQty": 1,
+      "options": [
+        { "name": "Bacon", "price": 0 },
+        { "name": "Sausage Patties", "price": 0 },
+        { "name": "Liver Mush", "price": 0 },
+        { "name": "Beef Bologna", "price": 0 }
+      ]
+    },
+    {
+      "groupName": "Choice of Side",
+      "isInclude": false,
+      "minQty": 1,
+      "maxQty": 1,
+      "options": [
+        { "name": "Grits", "price": 0 },
+        { "name": "Hash Browns", "price": 0 },
+        { "name": "Home Fries", "price": 0 }
+      ]
+    }
+  ]
+}
+F) This applies to ANY combo menu, not just breakfast combos — pizza combos, burger combos, thali/set-meal combos, etc. Always decompose into "fixed inclusion" groups vs "choice" groups using rules A and B above, regardless of cuisine or category name.
+--------------------------------------------------
+10. MODIFIER PRIORITY RULE
+--------------------------------------------------
+1. If modifier applies only to one item → Item-Level Modifier.
+2. If modifier applies to entire category → Category-Level Modifier.
+3. If modifier applies to multiple categories → Shared Category-Level Modifier.
+4. If modifier option has sub-options → Nested Modifier Group.
+5. Never duplicate modifier groups.
+--------------------------------------------------
+11. FINAL STRUCTURE (STRICT FORMAT)
+--------------------------------------------------
+Return ONLY this JSON structure:
+{
+  "categories": [
+    {
+      "category": "",
+      "lstInvSize": true/false,
+      "lstInventoryModifiers": true/false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "",
+          "description": null,
+          "sizes": {},
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    }
+  ],
+  "modifierGroups": [
+    {
+      "groupName": "",
+      "type": "modifier",
+      "lstInvSize": true/false,
+      "options": [
+        {
+          "name": "",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        }
+      ]
+    }
+  ]
+}
+--------------------------------------------------
+12. STRICT RULES
+--------------------------------------------------
+- Do not skip any item.
+- Keep prices as numbers only (no "/- " suffix, no currency symbols).
+- Remove brackets and their content from item names.
+- Do not duplicate modifier groups.
+- Do not leave price at item level if a modifier group exists, UNLESS every option in that modifier group is equal-price/no-cost (see Section 4C) — in that case keep the item price and set option prices to 0.
+- If price count and modifier count mismatch, map sequentially; assign 0 to unpaired options.
+- Nested modifiers must reference parent modifier correctly.
+- If a field is not applicable, set it to null (NOT empty string "").
+- "sizeType" must be null unless it is "ONLY_MEDIUM".
+- "modifierGroup" at category or item level must be null when not applicable.
+- "prices" field in modifier options must be {} (empty object) when not applicable.
+- "itemType" must be "product" for every regular item, and "combo" only for bundled/combo items (see Section 9B).
+- "comboGroups" must be [] for "product" items, and fully populated (fixed + choice groups, see Section 9C) for "combo" items.
+- Do not create multiple items in a category that share the same name/description and differ only by a size/portion tier label — merge into one item with "sizes" instead (see Section 2C).
+- If the same item text appears in more than one category, classify and structure it identically everywhere (see Section 9B consistency rule).
+- Do not leave "description" blank or skip modifiers just because a category's serving note (e.g. "served with X or Y, and A or B") sits outside the item row — apply it to every item in the category per Section 6B.
+- Return ONLY valid JSON.
+- Do NOT add explanations.
+- Do NOT use markdown.
+- Do not miss any itam details recheck and found any things is missing add the item proper as per rule
+</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>```json
+{
+  "categories": [
+    {
+      "category": "Seafarers' All Day Specials",
+      "lstInvSize": true,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Seafarers' All Day Special",
+          "description": "Fish, chips and peas with bread &amp; butter plus a cup of tea, coffee or a soft drink!",
+          "sizes": {
+            "Mini": 10.50,
+            "Senior": 11.95,
+            "Regular": 12.95,
+            "XLarge": 14.95
+          },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Pie Special",
+      "lstInvSize": false,
+      "lstInventoryModifiers": true,
+      "sizeType": null,
+      "modifierGroup": "Pie Special Filling Modifiers",
+      "items": [
+        {
+          "name": "Pie Special",
+          "description": "A traditional chip shop pie served piping-hot with chips, peas and gravy, and a cup of tea or coffee or soft-drink.",
+          "sizes": {},
+          "price": 11.75,
+          "modifierGroup": "Pie Special Filling Modifiers",
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Scampi Specials",
+      "lstInvSize": true,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Scampi Specials",
+          "description": "Lightly breaded scampi, deep fried until golden brown, served with chips, peas, a cup of tea, coffee or soft-drink.",
+          "sizes": {
+            "Mini": 10.50,
+            "Senior": 11.95,
+            "Regular": 12.95,
+            "XL": 17.95
+          },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Crispy Shredded Chicken",
+      "lstInvSize": false,
+      "lstInventoryModifiers": true,
+      "sizeType": null,
+      "modifierGroup": "Crispy Shredded Chicken Flavour Modifiers",
+      "items": [
+        {
+          "name": "Crispy Shredded Chicken",
+          "description": "Served with chips and a side.",
+          "sizes": {},
+          "price": 11.75,
+          "modifierGroup": "Crispy Shredded Chicken Flavour Modifiers",
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Starters &amp; Small Plates",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Classic Prawn Cocktail",
+          "description": "Succulent prawns served on fresh, crisp Iceberg lettuce with classic Marie Rose sauce and brown bread &amp; butter.",
+          "sizes": {},
+          "price": 6.50,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Jalapeno Peppers &amp; Chilli",
+          "description": "Chilli Peppers covered in tasty breadcrumbs with a delicious cream cheese filling.",
+          "sizes": {},
+          "price": 5.25,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Lightly Dusted Calamari",
+          "description": "Squid with salad garnish &amp; mayo.",
+          "sizes": {},
+          "price": 6.50,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Battered Haggis &amp; Black Pudding",
+          "description": "Served with salad garnish.",
+          "sizes": {},
+          "price": 5.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Chicken Popcorn (15 pieces)",
+          "description": "With fresh salad garnish &amp; mayo.",
+          "sizes": {},
+          "price": 4.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Halloumi Fries",
+          "description": "Delicious Halloumi fries served with freshly prepared side salad.",
+          "sizes": {},
+          "price": 5.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Hot 'n' Kickin Chicken Wings",
+      "lstInvSize": true,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Hot 'n' Kickin Chicken Wings",
+          "description": "Share as an appetiser or go LARGE as a main course! Served with salad garnish &amp; choice of dips.",
+          "sizes": {
+            "5 pcs": 5.75,
+            "10 pcs": 8.95,
+            "15 pcs": 12.50
+          },
+          "price": null,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Add Fries",
+          "description": null,
+          "sizes": {},
+          "price": 3.00,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Seafood Dishes",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Fish &amp; Chips",
+          "description": "Straight-up fish &amp; chips. Unbeatable!",
+          "sizes": {},
+          "price": 9.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Battered Plaice &amp; Chips",
+          "description": "Succulent Plaice fillet, deep-fried to order in light crispy batter.",
+          "sizes": {},
+          "price": 11.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Battered Lemon Sole &amp; Chips",
+          "description": "Deep-fried in a light crispy batter.",
+          "sizes": {},
+          "price": 12.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Seafarer Fish Burger &amp; Chips",
+          "description": "Served with chips, salad &amp; Tartar sauce.",
+          "sizes": {},
+          "price": 9.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Battered Haddock",
+          "description": "Haddock fillet with mash, peas &amp; parsley sauce.",
+          "sizes": {},
+          "price": 10.50,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Fish Finger Butty, Chips &amp; Peas",
+          "description": "Served with house mushy peas and a choice of chips or skinny fries.",
+          "sizes": {},
+          "price": 8.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Fish Cakes, Chips &amp; Peas",
+          "description": "2 lightly breaded fishcakes served with chips &amp; and our house mushy peas.",
+          "sizes": {},
+          "price": 10.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Baked Salmon",
+          "description": "Baked to perfection, served with chips or creamy mash potatoes.",
+          "sizes": {},
+          "price": 12.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Seafarer Combos",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Extra Special Chip Combos",
+          "description": "Bacon &amp; Cheese Chips.",
+          "sizes": {},
+          "price": 4.75,
+          "modifierGroup": null,
+          "itemType": "combo",
+          "comboGroups": [
+            {
+              "groupName": "Included",
+              "isInclude": true,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Bacon &amp; Cheese Chips", "price": 0 }
+              ]
+            }
+          ]
+        },
+        {
+          "name": "Classic 'Chicken In A Basket'",
+          "description": "A half oven cooked chicken served with chips or skinny fries and one side dish.",
+          "sizes": {},
+          "price": 11.75,
+          "modifierGroup": null,
+          "itemType": "combo",
+          "comboGroups": [
+            {
+              "groupName": "Chicken",
+              "isInclude": true,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Half Oven Cooked Chicken", "price": 0 }
+              ]
+            },
+            {
+              "groupName": "Choice of Fries",
+              "isInclude": false,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Chips", "price": 0 },
+                { "name": "Skinny Fries", "price": 0 }
+              ]
+            },
+            {
+              "groupName": "Side Dish",
+              "isInclude": true,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "One Side Dish", "price": 0 }
+              ]
+            }
+          ]
+        },
+        {
+          "name": "Oceans 2",
+          "description": "Mini fish, fishcake, chips and peas.",
+          "sizes": {},
+          "price": 10.95,
+          "modifierGroup": null,
+          "itemType": "combo",
+          "comboGroups": [
+            {
+              "groupName": "Included",
+              "isInclude": true,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Mini Fish, Fishcake, Chips and Peas", "price": 0 }
+              ]
+            }
+          ]
+        },
+        {
+          "name": "Tex Mex Platter",
+          "description": "Homemade Chilli Con Carne, spicy chicken wings, Jalapeno poppers, cheese, Pitta bread with chips or rice.",
+          "sizes": {},
+          "price": 14.75,
+          "modifierGroup": null,
+          "itemType": "combo",
+          "comboGroups": [
+            {
+              "groupName": "Included",
+              "isInclude": true,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Homemade Chilli Con Carne, Spicy Chicken Wings, Jalapeno Poppers, Cheese, Pitta Bread", "price": 0 }
+              ]
+            },
+            {
+              "groupName": "Choice of Side",
+              "isInclude": false,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Chips", "price": 0 },
+                { "name": "Rice", "price": 0 }
+              ]
+            }
+          ]
+        },
+        {
+          "name": "Fishbowl Combo",
+          "description": "Battered Haddock pieces, fish fingers &amp; Scampi. Served with chips or skinny fries.",
+          "sizes": {},
+          "price": 11.95,
+          "modifierGroup": null,
+          "itemType": "combo",
+          "comboGroups": [
+            {
+              "groupName": "Included",
+              "isInclude": true,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Battered Haddock Pieces, Fish Fingers &amp; Scampi", "price": 0 }
+              ]
+            },
+            {
+              "groupName": "Choice of Fries",
+              "isInclude": false,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Chips", "price": 0 },
+                { "name": "Skinny Fries", "price": 0 }
+              ]
+            }
+          ]
+        },
+        {
+          "name": "Boneless Chicken Bowl Combo",
+          "description": "Chicken nuggets, southern fried chicken strips, chicken popcorn with chips or skinny fries.",
+          "sizes": {},
+          "price": 11.95,
+          "modifierGroup": null,
+          "itemType": "combo",
+          "comboGroups": [
+            {
+              "groupName": "Included",
+              "isInclude": true,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Chicken Nuggets, Southern Fried Chicken Strips, Chicken Popcorn", "price": 0 }
+              ]
+            },
+            {
+              "groupName": "Choice of Fries",
+              "isInclude": false,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Chips", "price": 0 },
+                { "name": "Skinny Fries", "price": 0 }
+              ]
+            }
+          ]
+        },
+        {
+          "name": "Seafarer Davy Jones' Locker",
+          "description": "Our 'Seafood Basket Combo' PLUS fish fingers, scampi, sea stars, chips and dips.",
+          "sizes": {},
+          "price": 14.95,
+          "modifierGroup": null,
+          "itemType": "combo",
+          "comboGroups": [
+            {
+              "groupName": "Included",
+              "isInclude": true,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Seafood Basket Combo, Fish Fingers, Scampi, Sea Stars, Chips and Dips", "price": 0 }
+              ]
+            }
+          ]
+        },
+        {
+          "name": "Seafarer Country Platter",
+          "description": "Deep-fried battered tasty black pudding and Haggis served with chips and baked beans.",
+          "sizes": {},
+          "price": 11.95,
+          "modifierGroup": null,
+          "itemType": "combo",
+          "comboGroups": [
+            {
+              "groupName": "Included",
+              "isInclude": true,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Deep-fried Battered Black Pudding and Haggis, Chips and Baked Beans", "price": 0 }
+              ]
+            }
+          ]
+        },
+        {
+          "name": "Seafood Basket Combo",
+          "description": "Panko coated squid rings, breaded butterfly prawns, crispy cod bites, salt and pepper squid chunks, battered Haddock strips served with chips or skinny fries.",
+          "sizes": {},
+          "price": 11.95,
+          "modifierGroup": null,
+          "itemType": "combo",
+          "comboGroups": [
+            {
+              "groupName": "Included",
+              "isInclude": true,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Panko Coated Squid Rings, Breaded Butterfly Prawns, Crispy Cod Bites, Salt and Pepper Squid Chunks, Battered Haddock Strips", "price": 0 }
+              ]
+            },
+            {
+              "groupName": "Choice of Fries",
+              "isInclude": false,
+              "minQty": 1,
+              "maxQty": 1,
+              "options": [
+                { "name": "Chips", "price": 0 },
+                { "name": "Skinny Fries", "price": 0 }
+              ]
+            }
+          ]
+        }
+      ]
+    },
+    {
+      "category": "Seafarers' Classic Mains",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Chilli Con Carne",
+          "description": "Rich Chilli Con Carne topped with grated cheese, with chips, salad garnish and bread &amp; butter.",
+          "sizes": {},
+          "price": 11.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Chicken Curry",
+          "description": "Served with chips, side salad and poppadom.",
+          "sizes": {},
+          "price": 11.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Bangers (2) &amp; Mash",
+          "description": "Served with peas or beans and gravy.",
+          "sizes": {},
+          "price": 8.50,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Classic 'Chicken in a Basket'",
+          "description": "A half oven cooked chicken served with chips or skinny fries and one side dish.",
+          "sizes": {},
+          "price": 11.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Vegetable Curry",
+          "description": "Served with rice or chips and poppadom.",
+          "sizes": {},
+          "price": 9.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Upgrade Your Fries",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Cheesy Fries or Sweet Potato Fries Upgrade",
+          "description": "Ask for Cheesy Fries or Sweet Potato Fries. Just £2.00 extra!",
+          "sizes": {},
+          "price": 2.00,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Sides",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Onion Rings",
+          "description": null,
+          "sizes": {},
+          "price": 2.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Hash Browns",
+          "description": null,
+          "sizes": {},
+          "price": 0.80,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Skinny Fries",
+          "description": null,
+          "sizes": {},
+          "price": 4.25,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    },
+    {
+      "category": "Seafarers' Kids Favourites",
+      "lstInvSize": false,
+      "lstInventoryModifiers": false,
+      "sizeType": null,
+      "modifierGroup": null,
+      "items": [
+        {
+          "name": "Fish &amp; Chips",
+          "description": "Small fish and chips.",
+          "sizes": {},
+          "price": 7.50,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Sea Stars &amp; Chips",
+          "description": "With peas or beans.",
+          "sizes": {},
+          "price": 6.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Jumbo Fish Finger &amp; Chips",
+          "description": "With peas or beans.",
+          "sizes": {},
+          "price": 6.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Fishcake &amp; Chips",
+          "description": "With peas or beans.",
+          "sizes": {},
+          "price": 6.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Scampi &amp; Chips",
+          "description": "With peas or beans.",
+          "sizes": {},
+          "price": 7.95,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "100% Aberdeen Angus Burger &amp; Chips",
+          "description": "Succulent 100% Aberdeen Angus burger.",
+          "sizes": {},
+          "price": 7.25,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Sausage (2) &amp; Chips",
+          "description": "With peas or beans.",
+          "sizes": {},
+          "price": 6.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Hot Dog &amp; Chips",
+          "description": "With peas or beans.",
+          "sizes": {},
+          "price": 6.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Bangers &amp; Mash",
+          "description": "With peas, beans or gravy.",
+          "sizes": {},
+          "price": 6.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Spam Fritters &amp; Chips",
+          "description": "2 fritters with peas or beans.",
+          "sizes": {},
+          "price": 6.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Chicken Popcorn &amp; Chips",
+          "description": "12 pieces with peas or beans.",
+          "sizes": {},
+          "price": 6.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        },
+        {
+          "name": "Chicken Nuggets &amp; Chips",
+          "description": "4 nuggets with peas or beans.",
+          "sizes": {},
+          "price": 6.75,
+          "modifierGroup": null,
+          "itemType": "product",
+          "comboGroups": []
+        }
+      ]
+    }
+  ],
+  "modifierGroups": [
+    {
+      "groupName": "Pie Special Filling Modifiers",
+      "type": "modifier",
+      "lstInvSize": false,
+      "options": [
+        {
+          "name": "Choice of Filling",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": "Pie Special Filling Options"
+        }
+      ]
+    },
+    {
+      "groupName": "Pie Special Filling Options",
+      "type": "modifier",
+      "lstInvSize": false,
+      "options": [
+        {
+          "name": "Steak",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Meat &amp; Potato",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Cheese &amp; Onion",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Meat Pie",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Steak Pudding",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        }
+      ]
+    },
+    {
+      "groupName": "Crispy Shredded Chicken Flavour Modifiers",
+      "type": "modifier",
+      "lstInvSize": false,
+      "options": [
+        {
+          "name": "Choice of Flavour",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": "Crispy Shredded Chicken Flavour Options"
+        }
+      ]
+    },
+    {
+      "groupName": "Crispy Shredded Chicken Flavour Options",
+      "type": "modifier",
+      "lstInvSize": false,
+      "options": [
+        {
+          "name": "Plain",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Salt &amp; Pepper",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        },
+        {
+          "name": "Salt &amp; Chilli",
+          "price": 0,
+          "prices": {},
+          "modifierGroup": null
+        }
+      ]
+    }
+  ]
+}
+```</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>